<commit_message>
further enterprise build scipr improvements
</commit_message>
<xml_diff>
--- a/Excel/Enterprises/Enterprise_PastureBeef_Template_WIP_v01.xlsx
+++ b/Excel/Enterprises/Enterprise_PastureBeef_Template_WIP_v01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\Enterprises\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E627771-0161-402E-9E77-45D4CEA4F452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1053A381-C60D-42E0-8CA4-FC755A77FDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="180" windowWidth="35640" windowHeight="18855" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="35745" windowHeight="18900" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -502,24 +502,8 @@
     <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_StandardReferenceWeights_Unit">_xlfn.LAMBDA("kg")</definedName>
     <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_StandardReferenceWeights_Variable">_xlfn.LAMBDA("SRWk")</definedName>
     <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_StandardReferenceWeights_Variation">_xlfn.LAMBDA("VARIATION ON SOURCE: Split ACT and NSW into separate rows. Added 'State abbreviation' column to aid lookup.")</definedName>
-    <definedName name="Step1">#REF!</definedName>
-    <definedName name="Step2">#REF!</definedName>
-    <definedName name="Step3">#REF!</definedName>
-    <definedName name="VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_Result_Method1">#REF!</definedName>
-    <definedName name="VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_Result_Method2">#REF!</definedName>
-    <definedName name="VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_Result_Method1">#REF!</definedName>
-    <definedName name="VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_Result_Method2">#REF!</definedName>
-    <definedName name="VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_Result_Method1">#REF!</definedName>
-    <definedName name="VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_Result_Method2">#REF!</definedName>
-    <definedName name="VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_Result_Method1">#REF!</definedName>
-    <definedName name="VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_Result_Method2">#REF!</definedName>
     <definedName name="X_Cell_Enterprise_ProductionTimeframeEnd">'Input - Enterprise'!$E$19</definedName>
     <definedName name="X_Cell_Enterprise_ProductionTimeframeStart">'Input - Enterprise'!$E$18</definedName>
-    <definedName name="X_Cell_PastureBeef_Breed">#REF!</definedName>
-    <definedName name="X_Cell_PastureBeef_FencedWater">#REF!</definedName>
-    <definedName name="X_Cell_PastureBeef_GrazingIrrigationMethod">#REF!</definedName>
-    <definedName name="X_Cell_PastureBeef_GrazingProductionSystem">#REF!</definedName>
-    <definedName name="X_Cell_PastureBeef_ProductionRegion">#REF!</definedName>
     <definedName name="X_Cell_Site_AverageTemperature">'Input - Site'!$E$14</definedName>
     <definedName name="X_Cell_Site_ClimateZone">'Input - Site'!$E$20</definedName>
     <definedName name="X_Cell_Site_Elevation">'Input - Site'!$E$13</definedName>
@@ -536,18 +520,6 @@
     <definedName name="X_Cell_Site_TemperatureZone">'Input - Site'!$E$22</definedName>
     <definedName name="X_Cell_Site_TotalRainfall">'Input - Site'!$E$15</definedName>
     <definedName name="X_Cell_Site_WetOrDryClimateZone">'Input - Site'!$E$21</definedName>
-    <definedName name="X_Table_PastureBeef_CrudeProtein_Method1">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_CrudeProtein_Method2">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_DryMatterDigestibility_Method1">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_DryMatterDigestibility_Method2">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_Duration_Method1">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_Duration_Method2">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_Head_Method1">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_Head_Method2">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_Liveweight_Method1">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_Liveweight_Method2">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_LiveweightGain_Method1">#REF!</definedName>
-    <definedName name="X_Table_PastureBeef_LiveweightGain_Method2">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -607,7 +579,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="181">
   <si>
     <t>Home</t>
   </si>
@@ -618,9 +590,6 @@
     <t>APPENDICES</t>
   </si>
   <si>
-    <t>Emissions breakdown</t>
-  </si>
-  <si>
     <t>CALCULATIONS</t>
   </si>
   <si>
@@ -706,30 +675,6 @@
   </si>
   <si>
     <t>Percent manure applied to soil with no purpose (as waste)</t>
-  </si>
-  <si>
-    <t>Livestock sales</t>
-  </si>
-  <si>
-    <t>⚠️ Livestock sales are not automatically reflected in the herd movement data - you will need to manually adjust head count and average liveweight</t>
-  </si>
-  <si>
-    <t>Class</t>
-  </si>
-  <si>
-    <t>Sale date</t>
-  </si>
-  <si>
-    <t>Head sold</t>
-  </si>
-  <si>
-    <t>Average weight per head (kg)</t>
-  </si>
-  <si>
-    <t>Total liveweight sold</t>
-  </si>
-  <si>
-    <t>Bulls &gt; 1 year</t>
   </si>
   <si>
     <t>tonnes</t>
@@ -1222,6 +1167,15 @@
   </si>
   <si>
     <t>Input - Enterprise</t>
+  </si>
+  <si>
+    <t>Liveweight sold - method 1</t>
+  </si>
+  <si>
+    <t>Liveweight sold - method 2</t>
+  </si>
+  <si>
+    <t>percent</t>
   </si>
 </sst>
 </file>
@@ -4296,46 +4250,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6CBCD503-838A-4523-932C-9BA527D1C34C}" name="Table_Input_LivestockSales3" displayName="Table_Input_LivestockSales3" ref="D33:H35" totalsRowShown="0">
-  <autoFilter ref="D33:H35" xr:uid="{6CBCD503-838A-4523-932C-9BA527D1C34C}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2BFA511D-1E33-4FA7-9E53-155741FDE40A}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
+  <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{10611EAE-C98A-4772-A79C-DBC0DEE0D909}" name="Class"/>
-    <tableColumn id="2" xr3:uid="{C72E6C94-BA4D-4748-84FC-BCCF1BBBA7D6}" name="Sale date"/>
-    <tableColumn id="3" xr3:uid="{BC87B559-6411-49E0-9FED-D9EC6CFBBD83}" name="Head sold"/>
-    <tableColumn id="4" xr3:uid="{F08DE3C5-21CB-42C6-A868-7EFDDF741BF4}" name="Average weight per head (kg)"/>
-    <tableColumn id="5" xr3:uid="{9F84455A-39E1-4212-B9E8-759D853A4C96}" name="Total liveweight sold" dataCellStyle="Input number general calculated">
-      <calculatedColumnFormula>F34*G34</calculatedColumnFormula>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{A7717A66-4BDA-43C0-BFCD-4A6F29AEE8A3}" name="State/Territory">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Editable table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{EC0B98FF-3B1A-4F33-9028-A6B26A7E6CE4}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
-  <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{BBC50AC7-FEC1-431E-AD41-7CB9E130FE72}" name="Leaching Zone">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{D6D2A619-26C3-4096-9C5E-261DB4783E3F}" name="Common Name">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{ED997B4B-69AA-458D-AD94-F4C79A1B94D0}" name="Leaching criteria">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{8F8F275A-708B-458E-9ABF-5295B622DDF7}" name="Abbreviation">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{C1B321B1-DD2B-4EC5-AE20-D47C87F02BBF}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D153:E158" totalsRowShown="0">
   <autoFilter ref="D153:E158" xr:uid="{133D42B0-F6D2-470A-858A-37E6A7F5EC2B}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4353,7 +4289,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{14C890C4-4A77-40EC-A6C1-19C0895BD309}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
   <autoFilter ref="D134:E136" xr:uid="{308E99BE-FE1F-47A4-B2CA-97217277C4E9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4371,7 +4307,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{6BB36C9A-81C9-4008-9621-02E7765F4217}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D186:H199" totalsRowShown="0">
   <autoFilter ref="D186:H199" xr:uid="{D41FBEA4-8379-4DF7-A068-BF94D364F1A2}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4401,7 +4337,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{81046769-5E78-4435-8902-BE2F7ED271E9}" name="Table_SourceData_FracWETIrrigation" displayName="Table_SourceData_FracWETIrrigation" ref="D142:E147" totalsRowShown="0">
   <autoFilter ref="D142:E147" xr:uid="{1F48CA34-50DE-46D5-B32A-BB3A1E818E37}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4419,7 +4355,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{0D2D24A9-44B5-40A8-9D93-5D127038E490}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
   <autoFilter ref="D206:E208" xr:uid="{D5BE3F89-D70E-4C53-A71C-E756622DEF38}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4437,7 +4373,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{E20A54E0-06E3-423D-998B-2E4A7C9A48F2}" name="Table_SourceData_Common_MonthToSeason" displayName="Table_SourceData_Common_MonthToSeason" ref="D212:E224" totalsRowShown="0">
   <autoFilter ref="D212:E224" xr:uid="{97796C3A-D95E-4077-AA20-A8FE4145DAAD}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4455,7 +4391,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{06A63BFC-1602-47C1-AF55-49AA6B4633CD}" name="Table_SourceData_Common_MCFTemperatureZone" displayName="Table_SourceData_Common_MCFTemperatureZone" ref="D231:S250" totalsRowShown="0">
   <autoFilter ref="D231:S250" xr:uid="{1D72DD9B-C8FA-48F4-9A11-20231FF87B5A}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4529,7 +4465,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{949FFD0F-1699-4700-8323-CF2162C2663F}" name="Table_SourceData_Common_EFOrganicFertCropResidues" displayName="Table_SourceData_Common_EFOrganicFertCropResidues" ref="D257:E259" totalsRowShown="0">
   <autoFilter ref="D257:E259" xr:uid="{56E01C14-1BB8-4015-9158-4CEB4D3B605C}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4548,28 +4484,6 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2BFA511D-1E33-4FA7-9E53-155741FDE40A}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
-  <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{A7717A66-4BDA-43C0-BFCD-4A6F29AEE8A3}" name="State/Territory">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{D6D2A619-26C3-4096-9C5E-261DB4783E3F}" name="Common Name">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="3" xr3:uid="{8F8F275A-708B-458E-9ABF-5295B622DDF7}" name="Abbreviation">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A251EF82-BC21-4875-B405-6D0F230C2B8D}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
   <autoFilter ref="D20:D30" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4583,7 +4497,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{3F15B4B0-BD4E-4903-9096-ED3FE0A9167C}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
   <autoFilter ref="D36:E43" xr:uid="{B8E87A66-3E41-4AD3-925D-01EE21B43D7A}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4601,7 +4515,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{66C67C36-18E1-4B8A-BFF1-35CF3DC4AC81}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
   <autoFilter ref="D47:H54" xr:uid="{C1F562BB-DAA6-45BB-951A-7BAFA5B64B45}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4631,7 +4545,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{1D6C8105-982C-4B9F-A603-F884FE56E1B4}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
   <autoFilter ref="D89:S97" xr:uid="{5A437AE9-7724-4CF2-ACCF-291078682FB9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4705,7 +4619,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D228FD2E-DAAA-4D4F-BEFF-0E68A1F33AA0}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
   <autoFilter ref="D63:E77" xr:uid="{3597E019-B21E-4B76-BCC8-D02D497BCFA9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4723,7 +4637,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{E436A27C-11D9-4092-B110-DE3B0C7D7A9C}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
   <autoFilter ref="D109:G112" xr:uid="{AB16FEAB-AB03-45E1-BBD4-66D29CD412DF}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4749,7 +4663,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{AA9D31FA-C10A-401A-A990-FD7418530E07}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
   <autoFilter ref="D119:G121" xr:uid="{E08772F3-2E8C-40A8-B755-08A5BBDF4130}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -4769,6 +4683,24 @@
     </tableColumn>
     <tableColumn id="4" xr3:uid="{EDCA589F-5D6E-4F25-A934-864B94D632CD}" name="Max rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{EC0B98FF-3B1A-4F33-9028-A6B26A7E6CE4}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
+  <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{BBC50AC7-FEC1-431E-AD41-7CB9E130FE72}" name="Leaching Zone">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{ED997B4B-69AA-458D-AD94-F4C79A1B94D0}" name="Leaching criteria">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -4998,7 +4930,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="941" row="4">
+  <wetp:taskpane dockstate="right" visibility="0" width="565" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -5064,7 +4996,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -5092,8 +5024,9 @@
         <v>Results</v>
       </c>
       <c r="C4" s="9"/>
-      <c r="D4" s="2" t="s">
-        <v>3</v>
+      <c r="D4" s="2" t="str">
+        <f>"Emissions breakdown for activities running between " &amp; TEXT(X_Cell_Site_StartDate, "dd mmmm yyyy") &amp; " and " &amp; TEXT('Input - Enterprise'!E13, "dd mmmm yyyy")</f>
+        <v>Emissions breakdown for activities running between 01 January 2024 and 31 December 2024</v>
       </c>
       <c r="E4" s="11"/>
       <c r="F4" s="11"/>
@@ -5121,22 +5054,22 @@
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="G6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" s="21" t="s">
+      <c r="I6" s="21" t="s">
         <v>12</v>
-      </c>
-      <c r="I6" s="21" t="s">
-        <v>13</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="9"/>
@@ -5148,7 +5081,7 @@
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="1" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="E7" s="19" t="e" cm="1">
         <f t="array" ref="E7">VEERG_3_2_1_1__1_TotalAnnualMethaneFromEntericFermentation_Result_Method1</f>
@@ -5159,12 +5092,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G7" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="H7" s="19" t="e" cm="1">
+        <f t="array" ref="H7">Common_Equations.Common_ConvertCH4ToCO2e(E7,_xlfn.XLOOKUP("CH4", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I7" s="19" t="e" cm="1">
+        <f t="array" ref="I7">Common_Equations.Common_ConvertCH4ToCO2e(F7,_xlfn.XLOOKUP("CH4", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J7" s="16" t="s">
         <v>8</v>
-      </c>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="16" t="s">
-        <v>9</v>
       </c>
       <c r="K7" s="9"/>
     </row>
@@ -5175,21 +5114,29 @@
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
+        <v>14</v>
+      </c>
+      <c r="E8" s="19" t="e" cm="1">
+        <f t="array" ref="E8">VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_Result_Method1</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="F8" s="19" t="e" cm="1">
+        <f t="array" ref="F8">VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_Result_Method2</f>
+        <v>#NAME?</v>
+      </c>
       <c r="G8" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="H8" s="19" t="e" cm="1">
+        <f t="array" ref="H8">Common_Equations.Common_ConvertCH4ToCO2e(E8,_xlfn.XLOOKUP("CH4", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I8" s="19" t="e" cm="1">
+        <f t="array" ref="I8">Common_Equations.Common_ConvertCH4ToCO2e(F8,_xlfn.XLOOKUP("CH4", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J8" s="16" t="s">
         <v>8</v>
-      </c>
-      <c r="H8" s="19">
-        <v>1</v>
-      </c>
-      <c r="I8" s="19">
-        <v>2</v>
-      </c>
-      <c r="J8" s="16" t="s">
-        <v>9</v>
       </c>
       <c r="K8" s="9"/>
     </row>
@@ -5197,45 +5144,61 @@
       <c r="A9" s="5"/>
       <c r="C9" s="9"/>
       <c r="D9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
+        <v>16</v>
+      </c>
+      <c r="E9" s="19" t="e" cm="1">
+        <f t="array" ref="E9">VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_Result_Method1</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="F9" s="19" t="e" cm="1">
+        <f t="array" ref="F9">VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_Result_Method2</f>
+        <v>#NAME?</v>
+      </c>
       <c r="G9" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H9" s="19">
-        <v>2</v>
-      </c>
-      <c r="I9" s="19">
-        <v>3</v>
+        <v>15</v>
+      </c>
+      <c r="H9" s="19" t="e" cm="1">
+        <f t="array" ref="H9">Common_Equations.Common_ConvertN2OToCO2e(E9,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I9" s="19" t="e" cm="1">
+        <f t="array" ref="I9">Common_Equations.Common_ConvertN2OToCO2e(F9,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
       </c>
       <c r="J9" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K9" s="9"/>
     </row>
     <row r="10" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
+        <v>17</v>
+      </c>
+      <c r="E10" s="19" t="e" cm="1">
+        <f t="array" ref="E10">VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_Result_Method1</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="F10" s="19" t="e" cm="1">
+        <f t="array" ref="F10">VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_Result_Method2</f>
+        <v>#NAME?</v>
+      </c>
       <c r="G10" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" s="19">
-        <v>3</v>
-      </c>
-      <c r="I10" s="19">
-        <v>4</v>
+        <v>15</v>
+      </c>
+      <c r="H10" s="19" t="e" cm="1">
+        <f t="array" ref="H10">Common_Equations.Common_ConvertN2OToCO2e(E10,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I10" s="19" t="e" cm="1">
+        <f t="array" ref="I10">Common_Equations.Common_ConvertN2OToCO2e(F10,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
       </c>
       <c r="J10" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K10" s="9"/>
     </row>
@@ -5246,21 +5209,29 @@
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+        <v>18</v>
+      </c>
+      <c r="E11" s="19" t="e" cm="1">
+        <f t="array" ref="E11">VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_Result_Method1</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="F11" s="19" t="e" cm="1">
+        <f t="array" ref="F11">VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_Result_Method2</f>
+        <v>#NAME?</v>
+      </c>
       <c r="G11" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H11" s="19">
-        <v>4</v>
-      </c>
-      <c r="I11" s="19">
-        <v>5</v>
+        <v>15</v>
+      </c>
+      <c r="H11" s="19" t="e" cm="1">
+        <f t="array" ref="H11">Common_Equations.Common_ConvertN2OToCO2e(E11,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I11" s="19" t="e" cm="1">
+        <f t="array" ref="I11">Common_Equations.Common_ConvertN2OToCO2e(F11,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
       </c>
       <c r="J11" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K11" s="9"/>
     </row>
@@ -5271,7 +5242,7 @@
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="1" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="E12" s="19" t="e" cm="1">
         <f t="array" ref="E12">VEERG_5_1_1_1__1_InorganicFertiliserApplicationN2OEmissions_Result_Method1</f>
@@ -5282,12 +5253,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
+        <v>15</v>
+      </c>
+      <c r="H12" s="19" t="e" cm="1">
+        <f t="array" ref="H12">Common_Equations.Common_ConvertN2OToCO2e(E12,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I12" s="19" t="e" cm="1">
+        <f t="array" ref="I12">Common_Equations.Common_ConvertN2OToCO2e(F12,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J12" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K12" s="9"/>
     </row>
@@ -5298,7 +5275,7 @@
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="1" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E13" s="19" t="e" cm="1">
         <f t="array" ref="E13">VEERG_5_1_1_3__1_InorganicFertiliserApplicationCO2Emissions_Result_Method1</f>
@@ -5309,12 +5286,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
+        <v>149</v>
+      </c>
+      <c r="H13" s="19" t="e">
+        <f>E13</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I13" s="19" t="e">
+        <f>F13</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J13" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K13" s="9"/>
     </row>
@@ -5325,7 +5308,7 @@
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="1" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="E14" s="19" t="e" cm="1">
         <f t="array" ref="E14">VEERG_5_2_1_1__2_MassOfNitrogenInOrganicFertiliser_Result_Method1</f>
@@ -5336,12 +5319,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H14" s="19"/>
-      <c r="I14" s="19"/>
+        <v>15</v>
+      </c>
+      <c r="H14" s="19" t="e" cm="1">
+        <f t="array" ref="H14">Common_Equations.Common_ConvertN2OToCO2e(E14,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I14" s="19" t="e" cm="1">
+        <f t="array" ref="I14">Common_Equations.Common_ConvertN2OToCO2e(F14,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J14" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K14" s="9"/>
     </row>
@@ -5349,7 +5338,7 @@
       <c r="A15" s="5"/>
       <c r="C15" s="9"/>
       <c r="D15" s="1" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="E15" s="19" t="e" cm="1">
         <f t="array" ref="E15">VEERG_5_3_1_1__1_LimeApplicationCO2Emissions_Result_Method1</f>
@@ -5360,12 +5349,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
+        <v>149</v>
+      </c>
+      <c r="H15" s="19" t="e">
+        <f>E15</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I15" s="19" t="e">
+        <f>F15</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J15" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K15" s="9"/>
     </row>
@@ -5375,7 +5370,7 @@
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="1" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E16" s="19" t="e" cm="1">
         <f t="array" ref="E16">VEERG_5_4_1_3__1_OrganicFertiliserAtmosphericDepositionN2OEmissions_Result_Method1</f>
@@ -5386,12 +5381,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
+        <v>15</v>
+      </c>
+      <c r="H16" s="19" t="e" cm="1">
+        <f t="array" ref="H16">Common_Equations.Common_ConvertN2OToCO2e(E16,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I16" s="19" t="e" cm="1">
+        <f t="array" ref="I16">Common_Equations.Common_ConvertN2OToCO2e(F16,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J16" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K16" s="9"/>
     </row>
@@ -5402,7 +5403,7 @@
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="1" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="E17" s="19" t="e" cm="1">
         <f t="array" ref="E17">VEERG_5_5_1_1__1_FertiliserLeachingAndRunoffN2OEmissions_result_Method1</f>
@@ -5413,12 +5414,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
+        <v>15</v>
+      </c>
+      <c r="H17" s="19" t="e" cm="1">
+        <f t="array" ref="H17">Common_Equations.Common_ConvertN2OToCO2e(E17,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I17" s="19" t="e" cm="1">
+        <f t="array" ref="I17">Common_Equations.Common_ConvertN2OToCO2e(F17,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J17" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K17" s="9"/>
     </row>
@@ -5429,7 +5436,7 @@
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="1" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="E18" s="19" t="e" cm="1">
         <f t="array" ref="E18">VEERG_6_2_1_1__1__NitrousOxideEmissionsFromPastureResidues_Result_Method1</f>
@@ -5440,12 +5447,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
+        <v>15</v>
+      </c>
+      <c r="H18" s="19" t="e" cm="1">
+        <f t="array" ref="H18">Common_Equations.Common_ConvertN2OToCO2e(E18,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I18" s="19" t="e" cm="1">
+        <f t="array" ref="I18">Common_Equations.Common_ConvertN2OToCO2e(F18,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J18" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K18" s="9"/>
     </row>
@@ -5456,7 +5469,7 @@
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="1" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="E19" s="19" t="e" cm="1">
         <f t="array" ref="E19">VEERG_6_3_1_1__1__LeachingAndRunoffEmissionsCropAndPastureResidue_PastureOnly_Result_Method1</f>
@@ -5467,12 +5480,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
+        <v>15</v>
+      </c>
+      <c r="H19" s="19" t="e" cm="1">
+        <f t="array" ref="H19">Common_Equations.Common_ConvertN2OToCO2e(E19,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I19" s="19" t="e" cm="1">
+        <f t="array" ref="I19">Common_Equations.Common_ConvertN2OToCO2e(F19,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J19" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K19" s="9"/>
     </row>
@@ -5483,7 +5502,7 @@
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="1" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="E20" s="19" t="e" cm="1">
         <f t="array" ref="E20">VEERG_8_1_1_1__1_FuelCombustionTransport_Result_CO2</f>
@@ -5494,19 +5513,25 @@
         <v>#NAME?</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
+        <v>149</v>
+      </c>
+      <c r="H20" s="19" t="e">
+        <f>E20</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I20" s="19" t="e">
+        <f>F20</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J20" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K20" s="9"/>
     </row>
     <row r="21" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="9"/>
       <c r="D21" s="1" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E21" s="19" t="e" cm="1">
         <f t="array" ref="E21">VEERG_8_1_1_1__1_FuelCombustionTransport_Result_CH4</f>
@@ -5517,12 +5542,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G21" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="H21" s="19" t="e" cm="1">
+        <f t="array" ref="H21">Common_Equations.Common_ConvertCH4ToCO2e(E21,_xlfn.XLOOKUP("CH4", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I21" s="19" t="e" cm="1">
+        <f t="array" ref="I21">Common_Equations.Common_ConvertCH4ToCO2e(F21,_xlfn.XLOOKUP("CH4", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J21" s="16" t="s">
         <v>8</v>
-      </c>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="16" t="s">
-        <v>9</v>
       </c>
       <c r="K21" s="9"/>
     </row>
@@ -5530,7 +5561,7 @@
       <c r="A22" s="5"/>
       <c r="C22" s="9"/>
       <c r="D22" s="1" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="E22" s="19" t="e" cm="1">
         <f t="array" ref="E22">VEERG_8_1_1_1__1_FuelCombustionTransport_Result_N2O</f>
@@ -5541,12 +5572,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
+        <v>15</v>
+      </c>
+      <c r="H22" s="19" t="e" cm="1">
+        <f t="array" ref="H22">Common_Equations.Common_ConvertN2OToCO2e(E22,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I22" s="19" t="e" cm="1">
+        <f t="array" ref="I22">Common_Equations.Common_ConvertN2OToCO2e(F22,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J22" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K22" s="9"/>
     </row>
@@ -5554,7 +5591,7 @@
       <c r="A23" s="5"/>
       <c r="C23" s="9"/>
       <c r="D23" s="1" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="E23" s="19" t="e" cm="1">
         <f t="array" ref="E23">VEERG_8_2_1_1__1_FuelCombustionStationary_Result_CO2</f>
@@ -5565,12 +5602,18 @@
         <v>#NAME?</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
+        <v>149</v>
+      </c>
+      <c r="H23" s="19" t="e">
+        <f>E23</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I23" s="19" t="e">
+        <f>F23</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J23" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K23" s="9"/>
     </row>
@@ -5578,7 +5621,7 @@
       <c r="A24" s="5"/>
       <c r="C24" s="9"/>
       <c r="D24" s="1" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="E24" s="19" t="e" cm="1">
         <f t="array" ref="E24">VEERG_8_2_1_1__1_FuelCombustionStationary_Result_CH4</f>
@@ -5589,19 +5632,25 @@
         <v>#NAME?</v>
       </c>
       <c r="G24" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="H24" s="19" t="e" cm="1">
+        <f t="array" ref="H24">Common_Equations.Common_ConvertCH4ToCO2e(E24,_xlfn.XLOOKUP("CH4", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I24" s="19" t="e" cm="1">
+        <f t="array" ref="I24">Common_Equations.Common_ConvertCH4ToCO2e(F24,_xlfn.XLOOKUP("CH4", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J24" s="16" t="s">
         <v>8</v>
-      </c>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
-      <c r="J24" s="16" t="s">
-        <v>9</v>
       </c>
       <c r="K24" s="9"/>
     </row>
     <row r="25" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="9"/>
       <c r="D25" s="1" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="E25" s="19" t="e" cm="1">
         <f t="array" ref="E25">VEERG_8_2_1_1__1_FuelCombustionStationary_Result_N2O</f>
@@ -5612,19 +5661,25 @@
         <v>#NAME?</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
+        <v>15</v>
+      </c>
+      <c r="H25" s="19" t="e" cm="1">
+        <f t="array" ref="H25">Common_Equations.Common_ConvertN2OToCO2e(E25,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I25" s="19" t="e" cm="1">
+        <f t="array" ref="I25">Common_Equations.Common_ConvertN2OToCO2e(F25,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J25" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K25" s="9"/>
     </row>
     <row r="26" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="9"/>
       <c r="D26" s="1" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="E26" s="19" t="e" cm="1">
         <f t="array" ref="E26">VEERG_14_1_1__1_LocationBasedScopeElectricityEmissions_Result_Method1</f>
@@ -5635,19 +5690,25 @@
         <v>#NAME?</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
+        <v>8</v>
+      </c>
+      <c r="H26" s="19" t="e">
+        <f>E26</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I26" s="19" t="e">
+        <f>F26</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J26" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K26" s="9"/>
     </row>
     <row r="27" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="9"/>
       <c r="D27" s="1" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="E27" s="19" t="e" cm="1">
         <f t="array" ref="E27">VEERG_14_1_2__1_MarketBasedScopeElectricityEmissionsVariation_Result_Method1</f>
@@ -5658,33 +5719,39 @@
         <v>#NAME?</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
+        <v>8</v>
+      </c>
+      <c r="H27" s="19" t="e">
+        <f>E27</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I27" s="19" t="e">
+        <f>F27</f>
+        <v>#NAME?</v>
+      </c>
       <c r="J27" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K27" s="9"/>
     </row>
     <row r="28" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C28" s="9"/>
       <c r="D28" s="15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
       <c r="G28" s="15"/>
-      <c r="H28" s="20">
+      <c r="H28" s="20" t="e">
         <f>SUM(H7:H27)</f>
-        <v>10</v>
-      </c>
-      <c r="I28" s="20">
+        <v>#NAME?</v>
+      </c>
+      <c r="I28" s="20" t="e">
         <f>SUM(I7:I27)</f>
-        <v>14</v>
+        <v>#NAME?</v>
       </c>
       <c r="J28" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K28" s="9"/>
     </row>
@@ -5724,7 +5791,7 @@
     <row r="32" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C32" s="9"/>
       <c r="D32" s="2" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
@@ -5751,7 +5818,7 @@
     <row r="34" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C34" s="9"/>
       <c r="D34" s="1" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -5775,13 +5842,13 @@
     <row r="36" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C36" s="9"/>
       <c r="D36" s="21" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="E36" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="21" t="s">
         <v>12</v>
-      </c>
-      <c r="F36" s="21" t="s">
-        <v>13</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="14"/>
@@ -5804,7 +5871,7 @@
         <v>Enter value</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H37" s="14"/>
       <c r="I37" s="9"/>
@@ -5816,16 +5883,16 @@
       <c r="D38" s="1" t="str">
         <v>01 Jan 2024 to 31 Dec 2024 (This reporting cycle)</v>
       </c>
-      <c r="E38" s="88">
+      <c r="E38" s="88" t="e">
         <f>IF(ISBLANK($D38), "", IF(ISNUMBER(SEARCH("reporting", $D38)), Result_Enterprise_Method1, "Enter value"))</f>
-        <v>10</v>
-      </c>
-      <c r="F38" s="88">
+        <v>#NAME?</v>
+      </c>
+      <c r="F38" s="88" t="e">
         <f>IF(ISBLANK($D38), "", IF(ISNUMBER(SEARCH("reporting", $D38)), Result_Enterprise_Method2, "Enter value"))</f>
-        <v>14</v>
+        <v>#NAME?</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H38" s="14"/>
       <c r="I38" s="9"/>
@@ -5846,7 +5913,7 @@
         <v>Enter value</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H39" s="14"/>
       <c r="I39" s="9"/>
@@ -5865,7 +5932,7 @@
         <v/>
       </c>
       <c r="G40" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H40" s="14"/>
       <c r="I40" s="9"/>
@@ -5884,7 +5951,7 @@
         <v/>
       </c>
       <c r="G41" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H41" s="14"/>
       <c r="I41" s="9"/>
@@ -5894,15 +5961,15 @@
     <row r="42" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C42" s="9"/>
       <c r="D42" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="E42" s="20">
+        <v>150</v>
+      </c>
+      <c r="E42" s="20" t="e">
         <f>SUM(E37:E41)</f>
-        <v>10</v>
-      </c>
-      <c r="F42" s="20">
+        <v>#NAME?</v>
+      </c>
+      <c r="F42" s="20" t="e">
         <f>SUM(F37:F41)</f>
-        <v>14</v>
+        <v>#NAME?</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
@@ -5935,7 +6002,7 @@
     <row r="45" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C45" s="9"/>
       <c r="D45" s="2" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -5959,10 +6026,10 @@
     <row r="47" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C47" s="9"/>
       <c r="D47" s="21" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
@@ -5981,7 +6048,7 @@
         <v>0.6</v>
       </c>
       <c r="F48" s="16" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
@@ -5998,7 +6065,7 @@
         <v>0.5</v>
       </c>
       <c r="F49" s="16" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
@@ -6012,10 +6079,10 @@
         <v>01 Jan 2025 to 31 Dec 2025</v>
       </c>
       <c r="E50" s="88" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="F50" s="16" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
@@ -6028,7 +6095,7 @@
       <c r="D51" s="1"/>
       <c r="E51" s="88"/>
       <c r="F51" s="16" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
@@ -6041,7 +6108,7 @@
       <c r="D52" s="1"/>
       <c r="E52" s="88"/>
       <c r="F52" s="16" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
@@ -6052,7 +6119,7 @@
     <row r="53" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C53" s="9"/>
       <c r="D53" s="15" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="E53" s="20">
         <f>SUM(E48:E51)</f>
@@ -6090,7 +6157,7 @@
     <row r="56" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C56" s="9"/>
       <c r="D56" s="2" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
@@ -6115,10 +6182,10 @@
       <c r="C58" s="9"/>
       <c r="D58" s="21"/>
       <c r="E58" s="21" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="F58" s="21" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
@@ -6129,15 +6196,15 @@
     <row r="59" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C59" s="9"/>
       <c r="D59" s="91" t="s">
-        <v>161</v>
-      </c>
-      <c r="E59" s="89">
+        <v>152</v>
+      </c>
+      <c r="E59" s="89" t="e">
         <f>E42-E53</f>
-        <v>8.9</v>
-      </c>
-      <c r="F59" s="89">
+        <v>#NAME?</v>
+      </c>
+      <c r="F59" s="89" t="e">
         <f>F42-E53</f>
-        <v>12.9</v>
+        <v>#NAME?</v>
       </c>
       <c r="G59" s="1"/>
       <c r="H59" s="1"/>
@@ -6159,106 +6226,106 @@
     <row r="61" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C61" s="9"/>
       <c r="D61" s="21" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="E61" s="21" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="F61" s="21" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="G61" s="21" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="H61" s="21" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="I61" s="21" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="J61" s="21" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="K61" s="9"/>
     </row>
     <row r="62" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C62" s="9"/>
       <c r="D62" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="F62" s="19">
         <f>'Input - Enterprise'!E22</f>
-        <v>9.5</v>
-      </c>
-      <c r="G62" s="19">
+        <v>0</v>
+      </c>
+      <c r="G62" s="19" t="e">
         <f>F62/(F62+F63)</f>
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H62" s="19">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H62" s="19" t="e">
         <f>($E$42/F62)*G62</f>
-        <v>0.83333333333333326</v>
-      </c>
-      <c r="I62" s="19">
+        <v>#NAME?</v>
+      </c>
+      <c r="I62" s="19" t="e">
         <f>($F$42/F62)*G62</f>
-        <v>1.1666666666666665</v>
+        <v>#NAME?</v>
       </c>
       <c r="J62" s="16" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="K62" s="9"/>
     </row>
     <row r="63" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C63" s="9"/>
       <c r="D63" s="1" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="F63" s="19">
-        <f>'Input - Enterprise'!E25*'Input - Enterprise'!E26</f>
-        <v>2.5</v>
-      </c>
-      <c r="G63" s="19">
+        <f>'Input - Enterprise'!E26*'Input - Enterprise'!E27</f>
+        <v>0</v>
+      </c>
+      <c r="G63" s="19" t="e">
         <f>F63/(F62+F63)</f>
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H63" s="19">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H63" s="19" t="e">
         <f>($E$42/F63)*G63</f>
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="I63" s="19">
+        <v>#NAME?</v>
+      </c>
+      <c r="I63" s="19" t="e">
         <f>($F$42/F63)*G63</f>
-        <v>1.1666666666666667</v>
+        <v>#NAME?</v>
       </c>
       <c r="J63" s="16" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="K63" s="9"/>
     </row>
     <row r="64" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C64" s="9"/>
       <c r="D64" s="1" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="F64" s="19">
-        <f>'Input - Enterprise'!E25*'Input - Enterprise'!E27</f>
-        <v>1.5</v>
+        <f>'Input - Enterprise'!E26*'Input - Enterprise'!E28</f>
+        <v>0</v>
       </c>
       <c r="G64" s="19" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="H64" s="19" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="I64" s="19" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="J64" s="9"/>
       <c r="K64" s="9"/>
@@ -6277,54 +6344,54 @@
     <row r="66" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C66" s="9"/>
       <c r="D66" s="1" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="F66" s="19">
-        <f>'Input - Enterprise'!E23</f>
-        <v>300</v>
+        <f>'Input - Enterprise'!E24</f>
+        <v>0</v>
       </c>
       <c r="G66" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="H66" s="19">
+        <v>145</v>
+      </c>
+      <c r="H66" s="19" t="e">
         <f>E59/F66</f>
-        <v>2.9666666666666668E-2</v>
+        <v>#NAME?</v>
       </c>
       <c r="I66" s="19" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="J66" s="16" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="K66" s="9"/>
     </row>
     <row r="67" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C67" s="9"/>
       <c r="D67" s="1" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="F67" s="19">
-        <f>'Input - Enterprise'!E24</f>
-        <v>310</v>
+        <f>'Input - Enterprise'!E25</f>
+        <v>0</v>
       </c>
       <c r="G67" s="19" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="H67" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="I67" s="19">
+        <v>145</v>
+      </c>
+      <c r="I67" s="19" t="e">
         <f>F59/F67</f>
-        <v>4.161290322580645E-2</v>
+        <v>#NAME?</v>
       </c>
       <c r="J67" s="16" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="K67" s="9"/>
     </row>
@@ -6578,7 +6645,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="40" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:24" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6636,7 +6703,7 @@
     </row>
     <row r="5" spans="1:24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D5" s="2" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="N5" s="43"/>
     </row>
@@ -6652,7 +6719,7 @@
         <v>Site</v>
       </c>
       <c r="D7" s="55" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="E7" s="56"/>
       <c r="F7" s="56"/>
@@ -6664,7 +6731,7 @@
         <v>Pasture Beef</v>
       </c>
       <c r="D8" s="58" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="E8" s="59"/>
       <c r="F8" s="59"/>
@@ -6679,16 +6746,16 @@
     </row>
     <row r="10" spans="1:24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="F10" s="28" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="N10" s="47"/>
     </row>
@@ -6698,13 +6765,13 @@
         <v>4.2.1.1-2 Methane</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="E11" s="24" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="F11" s="28" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="G11" s="1"/>
       <c r="N11" s="52"/>
@@ -6715,13 +6782,13 @@
         <v>4.2.1.3-4 Soil direct N2O</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="E12" s="24" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6730,13 +6797,13 @@
         <v>4.2.1.5-6 Soil atm. deposition</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="E13" s="46">
         <v>307.7</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="N13" s="54"/>
       <c r="O13" s="54"/>
@@ -6747,13 +6814,13 @@
         <v>4.2.1.7-8 Soil leach &amp; runoff</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="E14" s="46">
         <v>18</v>
       </c>
       <c r="F14" s="28" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="N14" s="54"/>
       <c r="O14" s="54"/>
@@ -6761,13 +6828,13 @@
     <row r="15" spans="1:24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="D15" s="1" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E15" s="46">
         <v>601</v>
       </c>
       <c r="F15" s="28" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="N15" s="54"/>
       <c r="O15" s="54"/>
@@ -6777,13 +6844,13 @@
         <v>2</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="E16" s="46">
         <v>1326</v>
       </c>
       <c r="F16" s="28" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="N16" s="54"/>
       <c r="O16" s="54"/>
@@ -6794,13 +6861,13 @@
         <v>Constants - Pasture Beef</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="E17" s="46">
         <v>7</v>
       </c>
       <c r="F17" s="28" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18" spans="1:25" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6809,7 +6876,7 @@
         <v>Constants - Livestock</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="E18" s="27">
         <f>E15/E16</f>
@@ -6823,7 +6890,7 @@
         <v>Constants - Common</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="E19" s="27" t="str">
         <f>Common_InputFunctions.Utility_LookupItemFromMinMax(E15,Table_SourceData_RainfallZones[Min rainfall],Table_SourceData_RainfallZones[Max rainfall],Table_SourceData_RainfallZones[Rainfall Zone])</f>
@@ -6838,7 +6905,7 @@
         <v>Acknowledgements</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="E20" s="27" t="str">
         <f>Common_InputFunctions.Utility_GetClimateZone(E14,E15,E17,E13,E18,Table_SourceData_ClimateZones[Min temp],Table_SourceData_ClimateZones[Max temp],Table_SourceData_ClimateZones[Min rainfall],Table_SourceData_ClimateZones[Max rainfall],Table_SourceData_ClimateZones[Min frost days],Table_SourceData_ClimateZones[Max frost days],Table_SourceData_ClimateZones[Min elevation],Table_SourceData_ClimateZones[Max elevation],Table_SourceData_ClimateZones[Min MAP:PET],Table_SourceData_ClimateZones[Max MAP:PET],Table_SourceData_ClimateZones[Climate zone])</f>
@@ -6851,7 +6918,7 @@
     <row r="21" spans="1:25" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21"/>
       <c r="D21" s="1" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="E21" s="27" t="str">
         <f>Common_InputFunctions.Utility_LookupValueInTable($E$20,Table_SourceData_WetDryZones[Climate zone],Table_SourceData_WetDryZones[Wet or Dry Zone])</f>
@@ -6863,7 +6930,7 @@
     <row r="22" spans="1:25" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="D22" s="1" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="E22" s="27" t="str">
         <f>Common_InputFunctions.Utility_LookupItemFromMinMax(E14,Table_SourceData_TemperatureZones[Min MAT],Table_SourceData_TemperatureZones[Max MAT],Table_SourceData_TemperatureZones[Temperature Zone])</f>
@@ -7327,7 +7394,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A30171F5-957D-4D10-AA21-0CE17EC217CD}">
-  <dimension ref="C1:J35"/>
+  <dimension ref="C1:J32"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -7341,7 +7408,7 @@
   <sheetData>
     <row r="1" spans="3:10" ht="25.5" x14ac:dyDescent="0.35">
       <c r="C1" s="40" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="D1" s="34"/>
       <c r="E1" s="34"/>
@@ -7373,7 +7440,7 @@
     </row>
     <row r="5" spans="3:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D5" s="2" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="E5" s="37"/>
       <c r="F5" s="37"/>
@@ -7387,20 +7454,20 @@
     </row>
     <row r="7" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D7" s="1" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="E7" s="46" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="F7" s="28"/>
       <c r="G7" s="37"/>
     </row>
     <row r="8" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D8" s="23" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="E8" s="46" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="F8" s="37"/>
       <c r="G8" s="37"/>
@@ -7413,7 +7480,7 @@
     </row>
     <row r="10" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D10" s="48" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="E10" s="49"/>
       <c r="F10" s="50"/>
@@ -7427,26 +7494,26 @@
     </row>
     <row r="12" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D12" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E12" s="26">
         <v>45292</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="G12" s="37"/>
     </row>
     <row r="13" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D13" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E13" s="53">
         <f>DATE(YEAR(E12)+1,MONTH(E12),DAY(E12))-1</f>
         <v>45657</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="G13" s="37"/>
     </row>
@@ -7456,181 +7523,130 @@
     </row>
     <row r="16" spans="3:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D16" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D18" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E18" s="26">
         <v>45231</v>
       </c>
       <c r="F18" s="28" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D19" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E19" s="26">
         <v>45747</v>
       </c>
       <c r="F19" s="28" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D20" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E20" s="27">
         <f>DATEDIF(E18,E19+1,"m")</f>
         <v>17</v>
       </c>
       <c r="F20" s="28" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D22" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E22" s="27">
-        <f>SUM(Table_Input_LivestockSales3[Total liveweight sold])*10^-3</f>
-        <v>9.5</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="E22" s="27"/>
       <c r="F22" s="28" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D23" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E23" s="27">
-        <v>300</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="E23" s="27"/>
       <c r="F23" s="28" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D24" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E24" s="27">
-        <v>310</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="E24" s="27"/>
       <c r="F24" s="28" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D25" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E25" s="27">
-        <v>5</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="E25" s="27"/>
       <c r="F25" s="28" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D26" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E26" s="30">
-        <v>0.5</v>
+        <v>28</v>
+      </c>
+      <c r="E26" s="27"/>
+      <c r="F26" s="28" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D27" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E27" s="30">
-        <v>0.3</v>
+        <v>0.5</v>
+      </c>
+      <c r="F27" s="28" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="28" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D28" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E28" s="31">
-        <f>100%-E26-E27</f>
+        <v>30</v>
+      </c>
+      <c r="E28" s="30">
+        <v>0.3</v>
+      </c>
+      <c r="F28" s="28" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="29" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D29" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E29" s="31">
+        <f>100%-E27-E28</f>
         <v>0.2</v>
       </c>
+      <c r="F29" s="28" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="31" spans="4:6" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="D31" s="2" t="s">
-        <v>33</v>
-      </c>
+      <c r="D31" s="2"/>
     </row>
     <row r="32" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D32" s="25" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="33" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D33" s="32" t="s">
-        <v>35</v>
-      </c>
-      <c r="E33" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="F33" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="G33" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="H33" s="32" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="34" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D34" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="E34" s="32">
-        <v>45566</v>
-      </c>
-      <c r="F34" s="32">
-        <v>10</v>
-      </c>
-      <c r="G34" s="32">
-        <v>500</v>
-      </c>
-      <c r="H34" s="27">
-        <f>F34*G34</f>
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="35" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D35" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="E35" s="32">
-        <v>45415</v>
-      </c>
-      <c r="F35" s="32">
-        <v>10</v>
-      </c>
-      <c r="G35" s="32">
-        <v>450</v>
-      </c>
-      <c r="H35" s="27">
-        <f>F35*G35</f>
-        <v>4500</v>
-      </c>
+      <c r="D32" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -7667,7 +7683,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="33" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:65" s="3" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -7710,13 +7726,13 @@
     <row r="6" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6"/>
       <c r="D6" s="32" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="F6" s="32" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -7867,7 +7883,7 @@
     <row r="20" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20"/>
       <c r="D20" s="32" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -7966,10 +7982,10 @@
     <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36"/>
       <c r="D36" s="32" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E36" s="32" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8062,19 +8078,19 @@
     </row>
     <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D47" s="32" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E47" s="32" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F47" s="32" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="G47" s="32" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="H47" s="32" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8264,10 +8280,10 @@
     <row r="62" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="63" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D63" s="32" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="E63" s="32" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
     </row>
     <row r="64" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8454,52 +8470,52 @@
     <row r="88" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="89" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D89" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="E89" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="F89" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="G89" s="32" t="s">
+        <v>48</v>
+      </c>
+      <c r="H89" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="I89" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="J89" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="K89" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="L89" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="E89" s="32" t="s">
+      <c r="M89" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="N89" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="F89" s="32" t="s">
+      <c r="O89" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="G89" s="32" t="s">
+      <c r="P89" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="H89" s="32" t="s">
+      <c r="Q89" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="I89" s="32" t="s">
+      <c r="R89" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="J89" s="32" t="s">
+      <c r="S89" s="32" t="s">
         <v>60</v>
-      </c>
-      <c r="K89" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="L89" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="M89" s="32" t="s">
-        <v>63</v>
-      </c>
-      <c r="N89" s="32" t="s">
-        <v>64</v>
-      </c>
-      <c r="O89" s="32" t="s">
-        <v>65</v>
-      </c>
-      <c r="P89" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q89" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="R89" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="S89" s="32" t="s">
-        <v>69</v>
       </c>
       <c r="T89" s="32"/>
     </row>
@@ -9086,16 +9102,16 @@
     <row r="108" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="109" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D109" s="32" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="E109" s="32" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="F109" s="32" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="G109" s="32" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="110" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -9180,16 +9196,16 @@
     </row>
     <row r="119" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D119" s="32" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="E119" s="32" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="F119" s="32" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="G119" s="32" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="BN119" s="34"/>
     </row>
@@ -9250,10 +9266,10 @@
     <row r="126" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="127" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D127" s="32" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="E127" s="32" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
     </row>
     <row r="128" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -9294,10 +9310,10 @@
     </row>
     <row r="134" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D134" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="E134" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
     </row>
     <row r="135" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -9380,10 +9396,10 @@
     </row>
     <row r="142" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D142" s="32" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E142" s="32" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="BN142" s="34"/>
     </row>
@@ -9467,10 +9483,10 @@
     </row>
     <row r="153" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D153" s="32" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E153" s="32" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="BC153" s="37"/>
       <c r="BD153" s="37"/>
@@ -9740,19 +9756,19 @@
     </row>
     <row r="186" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D186" s="32" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="E186" s="32" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="F186" s="32" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="G186" s="32" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="H186" s="32" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="187" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -10067,10 +10083,10 @@
     </row>
     <row r="206" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D206" s="32" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="E206" s="32" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
     </row>
     <row r="207" spans="4:8" x14ac:dyDescent="0.25">
@@ -10101,10 +10117,10 @@
     </row>
     <row r="212" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D212" s="32" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E212" s="32" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
     </row>
     <row r="213" spans="4:5" x14ac:dyDescent="0.25">
@@ -10247,52 +10263,52 @@
     </row>
     <row r="231" spans="4:19" x14ac:dyDescent="0.25">
       <c r="D231" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="E231" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="F231" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="G231" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="H231" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="I231" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="J231" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="K231" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="L231" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="M231" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="E231" s="32" t="s">
+      <c r="N231" s="32" t="s">
         <v>91</v>
       </c>
-      <c r="F231" s="39" t="s">
+      <c r="O231" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="G231" s="32" t="s">
+      <c r="P231" s="32" t="s">
         <v>93</v>
       </c>
-      <c r="H231" s="32" t="s">
+      <c r="Q231" s="32" t="s">
         <v>94</v>
       </c>
-      <c r="I231" s="32" t="s">
+      <c r="R231" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="J231" s="32" t="s">
+      <c r="S231" s="32" t="s">
         <v>96</v>
-      </c>
-      <c r="K231" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="L231" s="32" t="s">
-        <v>98</v>
-      </c>
-      <c r="M231" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="N231" s="32" t="s">
-        <v>100</v>
-      </c>
-      <c r="O231" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="P231" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="Q231" s="32" t="s">
-        <v>103</v>
-      </c>
-      <c r="R231" s="32" t="s">
-        <v>104</v>
-      </c>
-      <c r="S231" s="32" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="232" spans="4:19" x14ac:dyDescent="0.25">
@@ -11575,10 +11591,10 @@
     </row>
     <row r="257" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D257" s="32" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="E257" s="32" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
     </row>
     <row r="258" spans="4:5" x14ac:dyDescent="0.25">
@@ -11627,15 +11643,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
@@ -11646,7 +11653,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -11841,19 +11848,20 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBvAHcAcwAsAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgACYAIABcACIAIAB0AG8AIABcACIAIAAmACAAZQBuAGQAcwBUAGUAeAB0ACAAJgAgAHQAYQBnACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBvAHcAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAA+ADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjACcAXAAiACAAJgAgAHMAaAAgACYAIABcACIAJwAhAFwAIgAgACYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgACYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADEALAAgADIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADMALAAgADQAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAATQBNAFMALAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFwAbgAgACAAIAAgACAAIAAgACAATQBFAEQASQBBAE4AKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgACYAIABcACIAIABcACIAIAAmACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAIABkAGEAdABhACAAdABoAGEAdAAgAGkAcwAgAGMAbwBtAG0AbwBuACAAYQBjAHIAbwBzAHMAIABhAGwAbAAgAGUAbgB0AGUAcgBwAHIAaQBzAGUAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQA6ACAATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXABuAE4ASQBSAF8AMgAwADIAMwBfAFYAbwBsADEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAFwAbgBwACAAPQAgAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlACAAKAAwAC4ANgA3ADgANAAgAGsAZwAvAG0AMwApAFwAbgBUAGEAawBlAG4AIABmAHIAbwBtACAAdABoAGUAIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAYQBuAGQAIABFAG4AZQByAGcAeQAgAFIAZQBwAG8AcgB0AGkAbgBnACAAXABuACgATQBlAGEAcwB1AHIAZQBtAGUAbgB0ACkAIABEAGUAdABlAHIAbQBpAG4AYQB0AGkAbwBuACAAMgAwADAAOABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwACAAPQAgAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AbQAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AcwAgADMALgBCAC4AMQBhAF8AMgAsACAAMwAuAEIALgAxAGMAXwAyACwAIAAzAC4AQgAuADMAXwAxACwAIAAzAC4AQgAuADQAZwBfADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgA2ADcAOAA0ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBcAG4AQwBnACAAPQAgADQANAAvADIAOAAgAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBnAE4AMgBPAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQANAAvADIAOAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBcAG4ARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAGEAcwBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMQBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAyAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgAFwAIgAxADYALwAxADIAXAAiACwAIAAxADYALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgAFwAIgA0ADQALwAyADgAXAAiACwAIAA0ADQALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AeABcACIALAAgAFwAIgA0ADYALwAxADQAXAAiACwAIAA0ADYALAAgADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AXAAiACwAIABcACIAMgA4AC8AMQAyAFwAIgAsACAAMgA4ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAIABMAGkAbQBlAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ATQBWAE8AQwBcACIALAAgAFwAIgAxADQALwAxADIAXAAiACwAIAAxADQALAAgADEAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAATgAyAE8AXABuAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAVwBQAE4AMgBPAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAGEAcwBcACIALAAgAFwAIgBDAE8AMgAtAGUAIABmAGEAYwB0AG8AcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAMgA2ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBGADQAXAAiACwAIAA2ADYAMwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAMgBGADYAXAAiACwAIAAxADIAMgAwADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBGADYAXAAiACwAIAAyADIAOAAwADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBGADMAXAAiACwAIAAxADcAMgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAdABhAHQAZQBzACAAYQBuAGQAIAB0AGUAcgByAGkAdABvAHIAaQBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlAC8AVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQwBvAG0AbQBvAG4AIABOAGEAbQBlAFwAIgAsACAAXAAiAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEMAYQBwAGkAdABhAGwAIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBBAEMAVABcACIALAAgAFwAIgBBAEMAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAQQBTAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBOAFQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAQgBTACAAUwB0AGEAdABpAHMAdABjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADQAIAAtACAAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABCAHUAcgBlAGEAdQAgAG8AZgAgAFMAdABhAHQAaQBzAHQAaQBjAHMAIAAoAEEAQgBTACkAIAAtACAAUwB0AGEAdABpAHMAdABpAGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAAMgAgAC0AIAAyADAAMgAxACAALQAgAFMAaABhAHAAZQBmAGkAbABlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAxACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEEAIAA0ACAATgBhAG0AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AG4AYgB1AHIAeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAG4AZAB1AHIAYQBoAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAASQBuAG4AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAFcAaABlAGEAdAAgAEIAZQBsAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABOAG8AcgB0AGgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAFMAbwB1AHQAaAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHcAZQB0ACAAYQBuAGQAIABkAHIAeQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMgA6ACAAVAByAGEAbgBzAGwAYQB0AGkAbgBnACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwAgAHQAbwAgAHcAZQB0ACAAYQBuAGQAIABkAHIAeQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAC0AIABDAGgAYQBuAGcAZQBkACAAJwBGAHIAeQAnACAAdABvACAAJwBEAHIAeQAnAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAD4AIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgADEAMAAwADAALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAD4AIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAPgAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAPgAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADAAIABDACAALQAgAGQiIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAPgAgADYAMAAwAG0AbQBcACIALAAgADYAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZCIgADYAMAAwAG0AbQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADYAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAWgBvAG4AZQBcACIALAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABjAHIAaQB0AGUAcgBpAGEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAG8AYwBjAHUAcgBzAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQA+AKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIAAnAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQAnACAAcgBvAHcALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGEAcwB0AGUAcgBpAHMAawBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAAnAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAJwAsACAAJwByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACcAIABhAG4AZAAgACcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkACcAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHUAcABsAGkAYwBhAHQAZQBkACAAJwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQAnACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgACcAQQByAGUAYQBzACAAYQByAGUAIABzAHUAYgBqAGUAYwB0ACAAdABvACAAbABlAGEAYwBoAGkAbgBnACAAKABpAC4AZQAuACwAIABpAG4AIAB0AGgAZQAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAKQAgAHcAaABlAG4ALgAuAC4AIAB0AGgAZQAgAGwAYQBuAGQAIABpAHMAIABpAHIAcgBpAGcAYQB0AGUAZAAgACgAZQB4AGMAZQBwAHQAIABkAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgApAC4AJwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAJwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAJwAgAHQAbwAgAHMAaQBuAGcAdQBsAGEAcgAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQAnACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAPAAxACAAbQBvAG4AdABoAFwAIgAsACAAXAAiAEQAZQBlAHAAIABMAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAATQBhAG4AdQByAGUAIAAoAHcAaQB0AGgALwB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAIABpAG4AdABvACAAcABlAGwAbABlAHQAaQB6AGUAZAAgAGYAZQByAHQAaQBsAGkAcwBlAHIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUALAAgAFIAYQBuAGcAZQAgAGEAbgBkACAAUABhAGQAZABvAGMAawAgACgAYwApACgAZAApAFwAIgAsACAAXAAiAE0AQQBUACAAcgBhAHcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIxADAAXAAiACwAIAAwAC4ANgA2ACwAIAAwAC4AMQAsACAAMAAuADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAxACwAIAAwAC4ANgA4ACwAIAAwAC4AMQAsACAAMAAuADEAMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADIALAAgADAALgA3ACwAIAAwAC4AMQAsACAAMAAuADEAMwAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADMALAAgADAALgA3ADEALAAgADAALgAxACwAIAAwAC4AMQA0ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEANAAsACAAMAAuADcAMwAsACAAMAAuADEALAAgADAALgAxADUALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANQAsACAAMAAuADcANAAsACAAMAAuADEALAAgADAALgAxADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADYALAAgADAALgA3ADUALAAgADAALgAxACwAIAAwAC4AMQA4ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA3ACwAIAAwAC4ANwA2ACwAIAAwAC4AMQAsACAAMAAuADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADgALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA5ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMAAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADYALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADEALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA5ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAyACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADMAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMwAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADQALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA1ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADQAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAMgA2ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADQANAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAMgA3ACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA0ADgALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIjIAOABcACIALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADUALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBEAGkAZwBlAHMAdABlAHIAIAAvACAAYwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAHMAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBQAGkAdAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAE0AQQBUACAAcgBhAHcAXAAiACAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIAByAG8AdwAgAG8AZgAgAE4ASQBSACAATQBNAEEAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABEAHUAcABsAGkAYwBhAHQAZQBkACAAJwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgACcATQBBAFQAIAByAGEAdwAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgACYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIAAmACAARQBGAE4AMgBPAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11864,7 +11872,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11883,10 +11891,18 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
convert stringified excel formula
</commit_message>
<xml_diff>
--- a/Excel/Enterprises/Enterprise_PastureBeef_Template_WIP_v01.xlsx
+++ b/Excel/Enterprises/Enterprise_PastureBeef_Template_WIP_v01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\Enterprises\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14DB445-5E0C-4BC9-BF83-D183E73330EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F1A04A5-E2C4-494A-8270-F8FF5809A45C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1215" yWindow="705" windowWidth="35745" windowHeight="18900" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -1189,19 +1189,19 @@
     <t>Percentage of income from manure sold</t>
   </si>
   <si>
-    <t>=SUM(Table_Input_LivestockSales348[Total liveweight sold])*10^-3</t>
-  </si>
-  <si>
     <t>=SUM(Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells('Input - Pasture Beef'!X_Table_PastureBeef_Head_Method1, 'Input - Pasture Beef'!X_Table_PastureBeef_Duration_Method1, 'Input - Pasture Beef'!X_Table_PastureBeef_LiveweightGain_Method1))*10^-3</t>
   </si>
   <si>
     <t>=SUM(Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells('Input - Pasture Beef'!X_Table_PastureBeef_Head_Method2, 'Input - Pasture Beef'!X_Table_PastureBeef_Duration_Method2, 'Input - Pasture Beef'!X_Table_PastureBeef_LiveweightGain_Method2))*10^-3</t>
   </si>
   <si>
-    <t>=SUM(Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells('Input - Pasture Beef'!X_Table_PastureBeef_Head_Method1, Input - Pasture Beef'!X_Table_PastureBeef_Duration_Method1, '4.2.1.1-2 Methane'!M1_Table_VS_j_k_l))*10^-3</t>
-  </si>
-  <si>
     <t>=SUM(Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells('Input - Pasture Beef'!X_Table_PastureBeef_Head_Method2, 'Input - Pasture Beef'!X_Table_PastureBeef_Duration_Method2, M2_Table_VS_j_k_l))*10^-3</t>
+  </si>
+  <si>
+    <t>=SUM(Table_Input_LivestockSales[Total liveweight sold])*10^-3</t>
+  </si>
+  <si>
+    <t>=SUM(Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells('Input - Pasture Beef'!X_Table_PastureBeef_Head_Method1, 'Input - Pasture Beef'!X_Table_PastureBeef_Duration_Method1, '4.2.1.1-2 Methane'!M1_Table_VS_j_k_l))*10^-3</t>
   </si>
 </sst>
 </file>
@@ -6284,7 +6284,7 @@
       </c>
       <c r="F62" s="19" t="str">
         <f>'Input - Enterprise'!E22</f>
-        <v>=SUM(Table_Input_LivestockSales348[Total liveweight sold])*10^-3</v>
+        <v>=SUM(Table_Input_LivestockSales[Total liveweight sold])*10^-3</v>
       </c>
       <c r="G62" s="19" t="e">
         <f>F62/(F62+F63)</f>
@@ -7592,7 +7592,7 @@
         <v>25</v>
       </c>
       <c r="E22" s="91" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="G22" s="27" t="s">
         <v>31</v>
@@ -7603,7 +7603,7 @@
         <v>26</v>
       </c>
       <c r="E23" s="91" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G23" s="27" t="s">
         <v>31</v>
@@ -7614,7 +7614,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="91" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G24" s="27" t="s">
         <v>31</v>
@@ -7625,7 +7625,7 @@
         <v>178</v>
       </c>
       <c r="E25" s="91" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G25" s="27" t="s">
         <v>31</v>
@@ -7636,7 +7636,7 @@
         <v>179</v>
       </c>
       <c r="E26" s="91" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G26" s="27" t="s">
         <v>31</v>
@@ -11696,19 +11696,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBvAHcAcwAsAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgACYAIABcACIAIAB0AG8AIABcACIAIAAmACAAZQBuAGQAcwBUAGUAeAB0ACAAJgAgAHQAYQBnACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBvAHcAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAA+ADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjACcAXAAiACAAJgAgAHMAaAAgACYAIABcACIAJwAhAFwAIgAgACYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgACYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADEALAAgADIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADMALAAgADQAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAATQBNAFMALAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFwAbgAgACAAIAAgACAAIAAgACAATQBFAEQASQBBAE4AKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgACYAIABcACIAIABcACIAIAAmACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAIABkAGEAdABhACAAdABoAGEAdAAgAGkAcwAgAGMAbwBtAG0AbwBuACAAYQBjAHIAbwBzAHMAIABhAGwAbAAgAGUAbgB0AGUAcgBwAHIAaQBzAGUAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQA6ACAATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXABuAE4ASQBSAF8AMgAwADIAMwBfAFYAbwBsADEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAFwAbgBwACAAPQAgAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlACAAKAAwAC4ANgA3ADgANAAgAGsAZwAvAG0AMwApAFwAbgBUAGEAawBlAG4AIABmAHIAbwBtACAAdABoAGUAIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAYQBuAGQAIABFAG4AZQByAGcAeQAgAFIAZQBwAG8AcgB0AGkAbgBnACAAXABuACgATQBlAGEAcwB1AHIAZQBtAGUAbgB0ACkAIABEAGUAdABlAHIAbQBpAG4AYQB0AGkAbwBuACAAMgAwADAAOABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwACAAPQAgAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AbQAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AcwAgADMALgBCAC4AMQBhAF8AMgAsACAAMwAuAEIALgAxAGMAXwAyACwAIAAzAC4AQgAuADMAXwAxACwAIAAzAC4AQgAuADQAZwBfADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgA2ADcAOAA0ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBcAG4AQwBnACAAPQAgADQANAAvADIAOAAgAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBnAE4AMgBPAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQANAAvADIAOAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBcAG4ARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAGEAcwBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMQBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAyAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgAFwAIgAxADYALwAxADIAXAAiACwAIAAxADYALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgAFwAIgA0ADQALwAyADgAXAAiACwAIAA0ADQALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AeABcACIALAAgAFwAIgA0ADYALwAxADQAXAAiACwAIAA0ADYALAAgADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AXAAiACwAIABcACIAMgA4AC8AMQAyAFwAIgAsACAAMgA4ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAIABMAGkAbQBlAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ATQBWAE8AQwBcACIALAAgAFwAIgAxADQALwAxADIAXAAiACwAIAAxADQALAAgADEAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAATgAyAE8AXABuAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAVwBQAE4AMgBPAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAGEAcwBcACIALAAgAFwAIgBDAE8AMgAtAGUAIABmAGEAYwB0AG8AcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAMgA2ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBGADQAXAAiACwAIAA2ADYAMwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAMgBGADYAXAAiACwAIAAxADIAMgAwADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBGADYAXAAiACwAIAAyADIAOAAwADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBGADMAXAAiACwAIAAxADcAMgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAdABhAHQAZQBzACAAYQBuAGQAIAB0AGUAcgByAGkAdABvAHIAaQBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlAC8AVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQwBvAG0AbQBvAG4AIABOAGEAbQBlAFwAIgAsACAAXAAiAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEMAYQBwAGkAdABhAGwAIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBBAEMAVABcACIALAAgAFwAIgBBAEMAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAQQBTAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBOAFQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAQgBTACAAUwB0AGEAdABpAHMAdABjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADQAIAAtACAAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABCAHUAcgBlAGEAdQAgAG8AZgAgAFMAdABhAHQAaQBzAHQAaQBjAHMAIAAoAEEAQgBTACkAIAAtACAAUwB0AGEAdABpAHMAdABpAGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAAMgAgAC0AIAAyADAAMgAxACAALQAgAFMAaABhAHAAZQBmAGkAbABlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAxACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEEAIAA0ACAATgBhAG0AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AG4AYgB1AHIAeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAG4AZAB1AHIAYQBoAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAASQBuAG4AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAFcAaABlAGEAdAAgAEIAZQBsAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABOAG8AcgB0AGgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAFMAbwB1AHQAaAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHcAZQB0ACAAYQBuAGQAIABkAHIAeQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMgA6ACAAVAByAGEAbgBzAGwAYQB0AGkAbgBnACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwAgAHQAbwAgAHcAZQB0ACAAYQBuAGQAIABkAHIAeQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAC0AIABDAGgAYQBuAGcAZQBkACAAJwBGAHIAeQAnACAAdABvACAAJwBEAHIAeQAnAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAD4AIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgADEAMAAwADAALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAD4AIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAPgAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAPgAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADAAIABDACAALQAgAGQiIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAPgAgADYAMAAwAG0AbQBcACIALAAgADYAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZCIgADYAMAAwAG0AbQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADYAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAWgBvAG4AZQBcACIALAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABjAHIAaQB0AGUAcgBpAGEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAG8AYwBjAHUAcgBzAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQA+AKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIAAnAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQAnACAAcgBvAHcALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGEAcwB0AGUAcgBpAHMAawBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAAnAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAJwAsACAAJwByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACcAIABhAG4AZAAgACcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkACcAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHUAcABsAGkAYwBhAHQAZQBkACAAJwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQAnACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgACcAQQByAGUAYQBzACAAYQByAGUAIABzAHUAYgBqAGUAYwB0ACAAdABvACAAbABlAGEAYwBoAGkAbgBnACAAKABpAC4AZQAuACwAIABpAG4AIAB0AGgAZQAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAKQAgAHcAaABlAG4ALgAuAC4AIAB0AGgAZQAgAGwAYQBuAGQAIABpAHMAIABpAHIAcgBpAGcAYQB0AGUAZAAgACgAZQB4AGMAZQBwAHQAIABkAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgApAC4AJwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAJwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAJwAgAHQAbwAgAHMAaQBuAGcAdQBsAGEAcgAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQAnACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAPAAxACAAbQBvAG4AdABoAFwAIgAsACAAXAAiAEQAZQBlAHAAIABMAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAATQBhAG4AdQByAGUAIAAoAHcAaQB0AGgALwB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAIABpAG4AdABvACAAcABlAGwAbABlAHQAaQB6AGUAZAAgAGYAZQByAHQAaQBsAGkAcwBlAHIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUALAAgAFIAYQBuAGcAZQAgAGEAbgBkACAAUABhAGQAZABvAGMAawAgACgAYwApACgAZAApAFwAIgAsACAAXAAiAE0AQQBUACAAcgBhAHcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIxADAAXAAiACwAIAAwAC4ANgA2ACwAIAAwAC4AMQAsACAAMAAuADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAxACwAIAAwAC4ANgA4ACwAIAAwAC4AMQAsACAAMAAuADEAMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADIALAAgADAALgA3ACwAIAAwAC4AMQAsACAAMAAuADEAMwAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADMALAAgADAALgA3ADEALAAgADAALgAxACwAIAAwAC4AMQA0ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEANAAsACAAMAAuADcAMwAsACAAMAAuADEALAAgADAALgAxADUALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANQAsACAAMAAuADcANAAsACAAMAAuADEALAAgADAALgAxADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADYALAAgADAALgA3ADUALAAgADAALgAxACwAIAAwAC4AMQA4ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA3ACwAIAAwAC4ANwA2ACwAIAAwAC4AMQAsACAAMAAuADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADgALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA5ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMAAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADYALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADEALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA5ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAyACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADMAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMwAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADQALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA1ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADQAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAMgA2ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADQANAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAMgA3ACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA0ADgALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIjIAOABcACIALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADUALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBEAGkAZwBlAHMAdABlAHIAIAAvACAAYwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAHMAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBQAGkAdAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAE0AQQBUACAAcgBhAHcAXAAiACAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIAByAG8AdwAgAG8AZgAgAE4ASQBSACAATQBNAEEAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABEAHUAcABsAGkAYwBhAHQAZQBkACAAJwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgACcATQBBAFQAIAByAGEAdwAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgACYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIAAmACAARQBGAE4AMgBPAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -11903,6 +11890,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBvAHcAcwAsAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgACYAIABcACIAIAB0AG8AIABcACIAIAAmACAAZQBuAGQAcwBUAGUAeAB0ACAAJgAgAHQAYQBnACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBvAHcAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAA+ADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjACcAXAAiACAAJgAgAHMAaAAgACYAIABcACIAJwAhAFwAIgAgACYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgACYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADEALAAgADIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADMALAAgADQAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAATQBNAFMALAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFwAbgAgACAAIAAgACAAIAAgACAATQBFAEQASQBBAE4AKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgACYAIABcACIAIABcACIAIAAmACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAIABkAGEAdABhACAAdABoAGEAdAAgAGkAcwAgAGMAbwBtAG0AbwBuACAAYQBjAHIAbwBzAHMAIABhAGwAbAAgAGUAbgB0AGUAcgBwAHIAaQBzAGUAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQA6ACAATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXABuAE4ASQBSAF8AMgAwADIAMwBfAFYAbwBsADEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAFwAbgBwACAAPQAgAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlACAAKAAwAC4ANgA3ADgANAAgAGsAZwAvAG0AMwApAFwAbgBUAGEAawBlAG4AIABmAHIAbwBtACAAdABoAGUAIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAYQBuAGQAIABFAG4AZQByAGcAeQAgAFIAZQBwAG8AcgB0AGkAbgBnACAAXABuACgATQBlAGEAcwB1AHIAZQBtAGUAbgB0ACkAIABEAGUAdABlAHIAbQBpAG4AYQB0AGkAbwBuACAAMgAwADAAOABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwACAAPQAgAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AbQAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AcwAgADMALgBCAC4AMQBhAF8AMgAsACAAMwAuAEIALgAxAGMAXwAyACwAIAAzAC4AQgAuADMAXwAxACwAIAAzAC4AQgAuADQAZwBfADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgA2ADcAOAA0ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBcAG4AQwBnACAAPQAgADQANAAvADIAOAAgAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBnAE4AMgBPAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQANAAvADIAOAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBcAG4ARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAGEAcwBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMQBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAyAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgAFwAIgAxADYALwAxADIAXAAiACwAIAAxADYALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgAFwAIgA0ADQALwAyADgAXAAiACwAIAA0ADQALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AeABcACIALAAgAFwAIgA0ADYALwAxADQAXAAiACwAIAA0ADYALAAgADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AXAAiACwAIABcACIAMgA4AC8AMQAyAFwAIgAsACAAMgA4ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAIABMAGkAbQBlAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ATQBWAE8AQwBcACIALAAgAFwAIgAxADQALwAxADIAXAAiACwAIAAxADQALAAgADEAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAATgAyAE8AXABuAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAVwBQAE4AMgBPAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAGEAcwBcACIALAAgAFwAIgBDAE8AMgAtAGUAIABmAGEAYwB0AG8AcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAMgA2ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBGADQAXAAiACwAIAA2ADYAMwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAMgBGADYAXAAiACwAIAAxADIAMgAwADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBGADYAXAAiACwAIAAyADIAOAAwADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBGADMAXAAiACwAIAAxADcAMgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAdABhAHQAZQBzACAAYQBuAGQAIAB0AGUAcgByAGkAdABvAHIAaQBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlAC8AVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQwBvAG0AbQBvAG4AIABOAGEAbQBlAFwAIgAsACAAXAAiAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEMAYQBwAGkAdABhAGwAIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBBAEMAVABcACIALAAgAFwAIgBBAEMAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAQQBTAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBOAFQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAQgBTACAAUwB0AGEAdABpAHMAdABjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADQAIAAtACAAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABCAHUAcgBlAGEAdQAgAG8AZgAgAFMAdABhAHQAaQBzAHQAaQBjAHMAIAAoAEEAQgBTACkAIAAtACAAUwB0AGEAdABpAHMAdABpAGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAAMgAgAC0AIAAyADAAMgAxACAALQAgAFMAaABhAHAAZQBmAGkAbABlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAxACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEEAIAA0ACAATgBhAG0AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AG4AYgB1AHIAeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAG4AZAB1AHIAYQBoAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAASQBuAG4AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAFcAaABlAGEAdAAgAEIAZQBsAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABOAG8AcgB0AGgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAFMAbwB1AHQAaAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHcAZQB0ACAAYQBuAGQAIABkAHIAeQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMgA6ACAAVAByAGEAbgBzAGwAYQB0AGkAbgBnACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwAgAHQAbwAgAHcAZQB0ACAAYQBuAGQAIABkAHIAeQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAC0AIABDAGgAYQBuAGcAZQBkACAAJwBGAHIAeQAnACAAdABvACAAJwBEAHIAeQAnAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAD4AIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgADEAMAAwADAALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAD4AIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAPgAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAPgAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADAAIABDACAALQAgAGQiIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAPgAgADYAMAAwAG0AbQBcACIALAAgADYAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZCIgADYAMAAwAG0AbQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADYAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAWgBvAG4AZQBcACIALAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABjAHIAaQB0AGUAcgBpAGEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAG8AYwBjAHUAcgBzAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQA+AKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIAAnAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQAnACAAcgBvAHcALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGEAcwB0AGUAcgBpAHMAawBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAAnAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAJwAsACAAJwByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACcAIABhAG4AZAAgACcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkACcAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHUAcABsAGkAYwBhAHQAZQBkACAAJwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQAnACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgACcAQQByAGUAYQBzACAAYQByAGUAIABzAHUAYgBqAGUAYwB0ACAAdABvACAAbABlAGEAYwBoAGkAbgBnACAAKABpAC4AZQAuACwAIABpAG4AIAB0AGgAZQAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAKQAgAHcAaABlAG4ALgAuAC4AIAB0AGgAZQAgAGwAYQBuAGQAIABpAHMAIABpAHIAcgBpAGcAYQB0AGUAZAAgACgAZQB4AGMAZQBwAHQAIABkAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgApAC4AJwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAJwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAJwAgAHQAbwAgAHMAaQBuAGcAdQBsAGEAcgAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQAnACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAPAAxACAAbQBvAG4AdABoAFwAIgAsACAAXAAiAEQAZQBlAHAAIABMAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAATQBhAG4AdQByAGUAIAAoAHcAaQB0AGgALwB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAIABpAG4AdABvACAAcABlAGwAbABlAHQAaQB6AGUAZAAgAGYAZQByAHQAaQBsAGkAcwBlAHIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUALAAgAFIAYQBuAGcAZQAgAGEAbgBkACAAUABhAGQAZABvAGMAawAgACgAYwApACgAZAApAFwAIgAsACAAXAAiAE0AQQBUACAAcgBhAHcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIxADAAXAAiACwAIAAwAC4ANgA2ACwAIAAwAC4AMQAsACAAMAAuADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAxACwAIAAwAC4ANgA4ACwAIAAwAC4AMQAsACAAMAAuADEAMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADIALAAgADAALgA3ACwAIAAwAC4AMQAsACAAMAAuADEAMwAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADMALAAgADAALgA3ADEALAAgADAALgAxACwAIAAwAC4AMQA0ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEANAAsACAAMAAuADcAMwAsACAAMAAuADEALAAgADAALgAxADUALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANQAsACAAMAAuADcANAAsACAAMAAuADEALAAgADAALgAxADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADYALAAgADAALgA3ADUALAAgADAALgAxACwAIAAwAC4AMQA4ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA3ACwAIAAwAC4ANwA2ACwAIAAwAC4AMQAsACAAMAAuADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADgALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA5ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMAAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADYALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADEALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA5ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAyACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADMAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMwAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADQALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA1ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADQAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAMgA2ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADQANAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAMgA3ACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA0ADgALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIjIAOABcACIALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADUALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBEAGkAZwBlAHMAdABlAHIAIAAvACAAYwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAHMAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBQAGkAdAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAE0AQQBUACAAcgBhAHcAXAAiACAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIAByAG8AdwAgAG8AZgAgAE4ASQBSACAATQBNAEEAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABEAHUAcABsAGkAYwBhAHQAZQBkACAAJwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgACcATQBBAFQAIAByAGEAdwAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgACYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIAAmACAARQBGAE4AMgBPAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -11915,22 +11915,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11949,6 +11933,22 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
fertiliser prod system for enterprises
</commit_message>
<xml_diff>
--- a/Excel/Enterprises/Enterprise_PastureBeef_Template_WIP_v01.xlsx
+++ b/Excel/Enterprises/Enterprise_PastureBeef_Template_WIP_v01.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\Enterprises\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F1A04A5-E2C4-494A-8270-F8FF5809A45C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5571C216-5A0E-4B64-A490-A74D7BACC52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="2070" yWindow="1515" windowWidth="36255" windowHeight="19140" activeTab="4" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
     <sheet name="Results" sheetId="13" r:id="rId2"/>
     <sheet name="Input - Site" sheetId="75" r:id="rId3"/>
     <sheet name="Input - Enterprise" sheetId="72" r:id="rId4"/>
-    <sheet name="Constants - Common" sheetId="74" r:id="rId5"/>
+    <sheet name="Input - Fert Prod System" sheetId="76" r:id="rId5"/>
+    <sheet name="Constants - Common" sheetId="74" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e">_xlfn.LAMBDA(_xlpm.E_CH4,_xlpm.GWP_CH4, _xlpm.E_CH4 * _xlpm.GWP_CH4)</definedName>
@@ -177,104 +178,6 @@
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Variable">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Variation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.";"Fixed typo - Changed 'Fry' to 'Dry'."}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="CommonCropping_InputFunctions.CommonCropping_CalculateFractionResidueRemoved">_xlfn.LAMBDA(_xlpm.TotalResidue,_xlpm.AmountRemoved, (_xlpm.AmountRemoved * 10 ^ 3) / (_xlpm.TotalResidue * 10 ^ 3))</definedName>
-    <definedName name="CommonCropping_InputFunctions.CommonCropping_CalculateHarvestIndex">_xlfn.LAMBDA(_xlpm.CropType,_xlpm.CropTypeArray,_xlpm.ResidueCropRatioArray, 1 / (1 + [0]!Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.CropType, _xlpm.CropTypeArray, _xlpm.ResidueCropRatioArray)))</definedName>
-    <definedName name="CommonCropping_InputFunctions.CommonCropping_CalculateResidueCropRatio">_xlfn.LAMBDA(_xlpm.HarvestIndex, (1 - _xlpm.HarvestIndex) / _xlpm.HarvestIndex)</definedName>
-    <definedName name="CommonCropping_InputFunctions.CommonCropping_GetFracWET">_xlfn.LAMBDA(_xlpm.LeachingZone,_xlpm.ProductionSystem,_xlpm.LeachingZoneLookup,_xlpm.LeachingZoneFracWETLookup,_xlpm.ProductionSystemLookup,_xlpm.ProductionSystemFracWETLookup, _xlfn.LET(_xlpm.LeachingZoneFracWET, [0]!Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.LeachingZone, _xlpm.LeachingZoneLookup, _xlpm.LeachingZoneFracWETLookup), _xlpm.ProductionSystemFracWET, [0]!Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.ProductionSystem, _xlpm.ProductionSystemLookup, _xlpm.ProductionSystemFracWETLookup), IF(_xlpm.LeachingZoneFracWET + _xlpm.ProductionSystemFracWET &gt; 0, 1, 0)))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.AverageLiveweightEndOfMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart,_xlpm.LiveweightAtStart,_xlpm.LiveweightGain, [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart) + [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightRemainingAtEndOfMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart, _xlpm.LiveweightAtStart, _xlpm.LiveweightGain))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.Livestock_LookupMCFState">_xlfn.LAMBDA(_xlpm.MMS,_xlpm.MMSArray,_xlpm.State,_xlpm.StateArray,_xlpm.ReturnArray, _xlfn.XLOOKUP(_xlpm.MMS, _xlpm.MMSArray, _xlfn.XLOOKUP(_xlpm.State, _xlpm.StateArray, _xlpm.ReturnArray)))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_AverageLiveweightAddedDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR([0]!CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass) / [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass), 0))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_GetMovementLiveweightGain">_xlfn.LAMBDA(_xlpm.LivestockClass,_xlpm.MovementDate, _xlfn.LET(_xlpm.ym, TEXT(_xlpm.MovementDate, "yyyymm"), IFERROR(INDEX(_xlfn._xlws.FILTER(#REF!, (TEXT(#REF!, "yyyymm") = _xlpm.ym) * (#REF! = _xlpm.LivestockClass)), 1), "")))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_HeadAddedDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_HeadAtEndOfMonth">_xlfn.LAMBDA(_xlpm.HeadAtStart,_xlpm.Month,_xlpm.LivestockClass, _xlpm.HeadAtStart + [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass) - [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadLostDuringMonth(_xlpm.Month, _xlpm.LivestockClass))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_HeadLostDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_HeadRemainingAtMonthEnd">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStartOfMonth, MAX(_xlpm.HeadAtStartOfMonth - [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadLostDuringMonth(_xlpm.Month, _xlpm.LivestockClass), 0))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_LiveweightAddedDuringMonth">_xlfn.LAMBDA(_xlpm.LivestockClass,_xlpm.MovementDate,_xlpm.WeightAtMovementDate,_xlpm.Head, IFERROR(_xlpm.Head * (_xlpm.WeightAtMovementDate + [0]!CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownDuringMonthPerHead(_xlpm.LivestockClass, _xlpm.MovementDate)), 0))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownDuringMonthPerHead">_xlfn.LAMBDA(_xlpm.LivestockClass,_xlpm.MovementDate, IFERROR([0]!CommonLivestock_InputFunctions.LivestockMovement_GetMovementLiveweightGain(_xlpm.LivestockClass, _xlpm.MovementDate) * CommonLivestock_InputFunctions.LivestockMovement_DaysMovementToMonthEnd(_xlpm.MovementDate), 0))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownFromMonthStartPerHead">_xlfn.LAMBDA(_xlpm.LivestockClass,_xlpm.Month, [0]!CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownDuringMonthPerHead(_xlpm.LivestockClass, EOMONTH(_xlpm.Month, -1) + 1))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownFromMonthStartTotal">_xlfn.LAMBDA(_xlpm.LivestockClass,_xlpm.Month,_xlpm.HeadAtStartOfMonth, [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadRemainingAtMonthEnd(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStartOfMonth) * [0]!CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownFromMonthStartPerHead(_xlpm.LivestockClass, _xlpm.Month))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownFromMovementDateTotal">_xlfn.LAMBDA(_xlpm.LivestockClass,_xlpm.MovementDate,_xlpm.Head, [0]!CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownDuringMonthPerHead(_xlpm.LivestockClass, _xlpm.MovementDate) * _xlpm.Head)</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightAddedDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart, [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionHeadAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart) * [0]!CommonLivestock_InputFunctions.LivestockMovement_AverageLiveweightAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightRemainingAtEndOfMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart,_xlpm.LiveweightAtStart,_xlpm.LiveweightGain, [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionHeadRemainingAtEndOfMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart) * CommonLivestock_InputFunctions.LivestockMovement_AverageLiveweightRemainingHead(_xlpm.Month, _xlpm.LiveweightAtStart, _xlpm.LiveweightGain))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_ProportionHeadAddedDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart, IFERROR(MIN(1, [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass) / [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAtEndOfMonth(_xlpm.HeadAtStart, _xlpm.Month, _xlpm.LivestockClass)), 0))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_ProportionHeadRemainingAtEndOfMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart, IFERROR(MIN(1, [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadRemainingAtMonthEnd(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart) / [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAtEndOfMonth(_xlpm.HeadAtStart, _xlpm.Month, _xlpm.LivestockClass)), 0))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightAddedDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightGrownDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
-    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightGrownDuringMonthAddedAndRemaining">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart, [0]!CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownFromMonthStartTotal(_xlpm.LivestockClass, _xlpm.Month, _xlpm.HeadAtStart) + [0]!CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightGrownDuringMonth(_xlpm.Month, _xlpm.LivestockClass))</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_FracLEACH_MS_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(8, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Production system","Emission factor";"Irrigated pasture",0.0059;"Irrigated crop",0.007;"Non-irrigated pasture",0.0018;"Non-irrigated crop",0.0041;"Sugar cane",0.0199;"Cotton",0.0053;"Horticulture",0.0064}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_FracLEACH_MS_Source">_xlfn.LAMBDA("National Inventory Report 2023 Volume 1: Equations 3.B.5a_3, 3.B.5c_3, 3.B.5d_3")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_FracLEACH_MS_Title">_xlfn.LAMBDA("Fraction of N lost through leaching and runoff")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_FracLEACH_MS_Unit">_xlfn.LAMBDA("Fraction")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_FracWETMMS_Data">_xlfn.LAMBDA(1)</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_FracWETMMS_Source">_xlfn.LAMBDA("National Inventory Report 2023 Volume 1: Equations 3.B.5a_3, 3.B.5c_3, 3.B.5d_3")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_FracWETMMS_Title">_xlfn.LAMBDA("Fraction of N available for leaching and runoff")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_FracWETMMS_Unit">_xlfn.LAMBDA("Fraction")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(19, 3, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Symbol","Manure management system","";"1","Anaerobic lagoon","Anaerobic lagoon (m=1)";"2","Liquid systems","Liquid systems (m=2)";"3","Daily spread","Daily spread (m=3)";"3a","Sump and dispersal system","Sump and dispersal system (m=3a)";"3b","Drains to paddock","Drains to paddock (m=3b)";"4","Solid storage","Solid storage (m=4)";"5","Drylot (feed pad)","Drylot (feed pad) (m=5)";"6","Composting (passive windrow)","Composting (passive windrow) (m=6)";"7","Digester / covered lagoons","Digester / covered lagoons (m=7)";"8","Deep litter","Deep litter (m=8)";"9","Pit storage","Pit storage (m=9)";"10","Poultry manure with bedding","Poultry manure with bedding (m=10)";"11","Poultry manure without bedding","Poultry manure without bedding (m=11)";"11a","Belt manure removal","Belt manure removal (m=11a)";"11b","Manure stored in house","Manure stored in house (m=11b)";"12","Direct processing","Direct processing (m=12)";"13","Direct application","Direct application (m=13)";"14","Pasture range and paddock","Pasture range and paddock (m=14)"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Source">_xlfn.LAMBDA("National Inventory Report 2023 Volume 1: Table 5.12")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Title">_xlfn.LAMBDA("Table 5.12 Additional symbols used in algorithms for manure related emissions")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Unit">_xlfn.LAMBDA("")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Vairable">_xlfn.LAMBDA("MMS")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_BeefCattle_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Source region";"Cattle, for manufacturing beef","Australia";"Cattle, for prime beef","NSW";"Cattle, weaners","NT";"","QLD";"","SA";"","TAS";"","VIC";"","WA"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_BeefCattle_Source">_xlfn.LAMBDA("Lifecycles. (2026). Greenhouse Gas Emission Intensities for Material Inputs to Australian Agriculture, Fisheries and Forestry. Version 48. doi 10.5281/zenodo.19656580")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_BeefCattle_Title">_xlfn.LAMBDA("Beef cattle products for scope 3")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_BeefCattle_Unit">_xlfn.LAMBDA("")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_BeefCattle_Vairable">_xlfn.LAMBDA("")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Chickens_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Source region";"Chickens","Australia"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Chickens_Source">_xlfn.LAMBDA("Lifecycles. (2026). Greenhouse Gas Emission Intensities for Material Inputs to Australian Agriculture, Fisheries and Forestry. Version 48. doi 10.5281/zenodo.19656580")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Chickens_Title">_xlfn.LAMBDA("Chickens products for scope 3")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Chickens_Unit">_xlfn.LAMBDA("")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Chickens_Vairable">_xlfn.LAMBDA("")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Dairycattle_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Source region";"Dairy cows","VIC"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Dairycattle_Source">_xlfn.LAMBDA("Lifecycles. (2026). Greenhouse Gas Emission Intensities for Material Inputs to Australian Agriculture, Fisheries and Forestry. Version 48. doi 10.5281/zenodo.19656580")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Dairycattle_Title">_xlfn.LAMBDA("Dairy cattle products for scope 3")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Dairycattle_Unit">_xlfn.LAMBDA("")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Dairycattle_Vairable">_xlfn.LAMBDA("")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Pigs_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Source region";"Pigs","Australia"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Pigs_Source">_xlfn.LAMBDA("Lifecycles. (2026). Greenhouse Gas Emission Intensities for Material Inputs to Australian Agriculture, Fisheries and Forestry. Version 48. doi 10.5281/zenodo.19656580")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Pigs_Title">_xlfn.LAMBDA("Pigs products for scope 3")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Pigs_Unit">_xlfn.LAMBDA("")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Pigs_Vairable">_xlfn.LAMBDA("")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Sheep_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(8, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Source region";"Sheep, for mutton","Australia";"Sheep, for prime lamb","NSW";"","QLD";"","SA";"","TAS";"","VIC";"","WA"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Sheep_Source">_xlfn.LAMBDA("Lifecycles. (2026). Greenhouse Gas Emission Intensities for Material Inputs to Australian Agriculture, Fisheries and Forestry. Version 48. doi 10.5281/zenodo.19656580")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Sheep_Title">_xlfn.LAMBDA("Sheep products for scope 3")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Sheep_Unit">_xlfn.LAMBDA("")</definedName>
-    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Sheep_Vairable">_xlfn.LAMBDA("")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__1_TotalAnnualMethaneFromEntericFermentation">_xlfn.LAMBDA(_xlpm.D_j,_xlpm.M_jkl,_xlpm.N_jkl, (_xlpm.D_j * _xlpm.M_jkl * _xlpm.N_jkl) * 10 ^ -3)</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__1_TotalAnnualMethaneFromEntericFermentation_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"D_j","number of days the animal is on the farm in each time-period","days","Input";"M_jkl","daily production of enteric methane in each time-period, class and subclass","kg CH4/head/day","Calculated from 3.2.1.1, (2)";"N_jkl","number of beef cattle in each time-period, class and subclass","head","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__1_TotalAnnualMethaneFromEntericFermentation_LatexEquation">_xlfn.LAMBDA("E_{enteric}=\sum_{j}\sum_{k}\sum_{l}(D_j\times M_{jkl}\times N_{jkl})\times 10^{-3}")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__1_TotalAnnualMethaneFromEntericFermentation_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__1_TotalAnnualMethaneFromEntericFermentation_Source">_xlfn.LAMBDA("VEERG 2026: 3.2.1.1, Equation (1)")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__1_TotalAnnualMethaneFromEntericFermentation_Title">_xlfn.LAMBDA("Total annual methane production from enteric fermentation in grazing beef cattle")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__1_TotalAnnualMethaneFromEntericFermentation_Unit">_xlfn.LAMBDA("t CH4")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__1_TotalAnnualMethaneFromEntericFermentation_Variable">_xlfn.LAMBDA("E_enteric")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__2_DailyEntericMethaneProduction">_xlfn.LAMBDA(_xlpm.I_jkl, 20.7 * _xlpm.I_jkl * 10 ^ -3)</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__2_DailyEntericMethaneProduction_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(1, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"I_jkl","dry matter intake","kg DM/head/day","Calculated from 3.2.1.1, (3)"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__2_DailyEntericMethaneProduction_LatexEquation">_xlfn.LAMBDA("M_{jkl}=20.7\times I_{jkl}\times 10^{-3}")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__2_DailyEntericMethaneProduction_NIRReference">_xlfn.LAMBDA("Charmley et al. (2015)")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__2_DailyEntericMethaneProduction_Source">_xlfn.LAMBDA("VEERG 2026: 3.2.1.1, Equation (2)")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__2_DailyEntericMethaneProduction_Title">_xlfn.LAMBDA("Daily production of enteric methane")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__2_DailyEntericMethaneProduction_Unit">_xlfn.LAMBDA("kg CH4/head/day")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__2_DailyEntericMethaneProduction_Variable">_xlfn.LAMBDA("M_jkl")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__3_FeedIntakeForGrazingBeef">_xlfn.LAMBDA(_xlpm.W_jkl,_xlpm.LWG_jkl,_xlpm.MA_jk45, (1.185 + 0.00454 * _xlpm.W_jkl - 0.0000026 * _xlpm.W_jkl ^ 2 + 0.315 * _xlpm.LWG_jkl) ^ 2 * _xlpm.MA_jk45)</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__3_FeedIntakeForGrazingBeef_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"W_jkl","liveweight (kg)","kg","Input";"LWG_jkl","live weight gain (kg/head/day)","kg/head/day","Input";"MA_jk45","additional intake for milk production in cows greater than 2 years","kg/head/day","Calculated from 3.2.1.1, (4)"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__3_FeedIntakeForGrazingBeef_LatexEquation">_xlfn.LAMBDA("I_{jkl}=(1.185+0.00454\times W_{jkl}-0.0000026\times W_{jkl}^{2}+0.315\times LWG_{jkl})^2\times MA_{jk=4,5}")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__3_FeedIntakeForGrazingBeef_NIRReference">_xlfn.LAMBDA("Minson and McDonald (1987)")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__3_FeedIntakeForGrazingBeef_Source">_xlfn.LAMBDA("VEERG 2026: 3.2.1.1, Equation (3)")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__3_FeedIntakeForGrazingBeef_Title">_xlfn.LAMBDA("Feed intake for grazing beef cattle")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__3_FeedIntakeForGrazingBeef_Unit">_xlfn.LAMBDA("kg DM/head/day")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__3_FeedIntakeForGrazingBeef_Variable">_xlfn.LAMBDA("I_jkl")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction">_xlfn.LAMBDA(_xlpm.LC_jk45,_xlpm.FA_jk45, (_xlpm.LC_jk45 * _xlpm.FA_jk45) + (1 - _xlpm.LC_jk45))</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"LC_jk45","proportion of cows greater than 1 year in calf in the season of calving expressed as a fraction","fraction","Input";"FA_jk45","feed adjustment value for lactating cows in the season of calving and the season immediately after calving expressed as a fraction","fraction","Constant";"b","breed of cattle","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction_ArgumentsVariation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"LC_jk45","proportion of cows greater than 1 year in calf in the season of calving expressed as a fraction","fraction","Input";"FA_jk45calv","feed adjustment value for lactating cows in the season of calving expressed as a fraction","fraction","Constant";"FA_jk45after","feed adjustment value for lactating cows in the season immediately after calving expressed as a fraction","fraction","Constant";"b","breed of cattle","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction_LatexEquation">_xlfn.LAMBDA("MA_{jk=4,5}=(LC_{jk=4,5}\times FA_{jk=4,5})+(1-LC_{jk=4,5})")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction_LatexEquationVariation">_xlfn.LAMBDA("MA_{jk=4,5}=((LC_{jk=4,5,calv}\times FA_{jk=4,5,calv})+(LC_{jk=4,5,prev}\times FA_{jk=4,5,after}))+(1-(LC_{jk=4,5,calv}+LC_{jk=4,5,prev}))")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction_Source">_xlfn.LAMBDA("VEERG 2026: 3.2.1.1, Equation (4)")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction_Title">_xlfn.LAMBDA("Additional intake for milk production in the season of calving and the season after calving")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction_Unit">_xlfn.LAMBDA("fraction")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction_Variable">_xlfn.LAMBDA("MA_jk45")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProduction_Variation">_xlfn.LAMBDA("VARIATION ON SOURCE: Expanded equation to account for season after calving, rather than doing the same equation twice for both seasons")</definedName>
-    <definedName name="EntericMethane_PastureBeef_Equations.VEERG_3_2_1_1__4_AdditionalIntakeForMilkProductionVariation">_xlfn.LAMBDA(_xlpm.LC_jk45calv,_xlpm.LC_jk45prev,_xlpm.FA_jk45calv,_xlpm.FA_jk45after, ((_xlpm.LC_jk45calv * _xlpm.FA_jk45calv) + (_xlpm.LC_jk45prev * _xlpm.FA_jk45after)) + (1 - (_xlpm.LC_jk45calv + _xlpm.LC_jk45prev)))</definedName>
     <definedName name="Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells">_xlfn.LAMBDA(_xlpm.range1,_xlpm.range2,_xlpm.range3, _xlfn.LET(_xlpm.numRows, ROWS(_xlpm.range1), _xlpm.numCols, COLUMNS(_xlpm.range1), _xlpm.result, _xlfn.MAKEARRAY(_xlpm.numRows, _xlpm.numCols, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, IF(ISNUMBER(INDEX(_xlpm.range1, _xlpm.r, _xlpm.c)), INDEX(_xlpm.range1, _xlpm.r, _xlpm.c), 0) * IF(ISNUMBER(INDEX(_xlpm.range2, _xlpm.r, _xlpm.c)), INDEX(_xlpm.range2, _xlpm.r, _xlpm.c), 0) * IF(ISNUMBER(INDEX(_xlpm.range3, _xlpm.r, _xlpm.c)), INDEX(_xlpm.range3, _xlpm.r, _xlpm.c), 0))), _xlpm.result))</definedName>
     <definedName name="getOverlappingReportingCycles">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingStartMonth,_xlpm.ReportingStartDay, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, _xlpm.ReportingStartMonth, _xlpm.d, _xlpm.ReportingStartDay, _xlpm.A, _xlpm.S - 364, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (DATE(_xlpm.ya, _xlpm.m, _xlpm.d) &lt; _xlpm.A), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1)))</definedName>
     <definedName name="Inoput_Cell_Livestock_antibiotics">#REF!</definedName>
@@ -299,124 +202,6 @@
     <definedName name="M1_Table_MA_j_k45">#REF!</definedName>
     <definedName name="M1_Table_VS_j_k_l">#REF!</definedName>
     <definedName name="M2_Table_I_j_k_l">#REF!</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement">_xlfn.LAMBDA(_xlpm.N_jkl,_xlpm.M_jklm,_xlpm.D_j, (_xlpm.N_jkl * _xlpm.M_jklm * _xlpm.D_j) * 10 ^ -3)</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"N_jkl","number of beef cattle in each time-period, class and subclass","head","Input";"M_jklm","methane production from manure in each time-period, class, subclass and MMS","kg/head/day","Calculated from 4.2.1.1 (2)";"D_j","number of days in each time-period for each input class","days","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_LatexEquation">_xlfn.LAMBDA("E_{CH4}=\sum_{j}\sum_{k}\sum_{l}\sum_{m}(N_{jkl}\times M_{jklm}\times D_j)\times 10^{-3}")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.1, Equation (1)")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_Title">_xlfn.LAMBDA("Total annual methane production from manure management for grazing beef cattle")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_Unit">_xlfn.LAMBDA("t CH4")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_Variable">_xlfn.LAMBDA("E_CH4")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__2_MethaneProductionFromManure">_xlfn.LAMBDA(_xlpm.VS_jkl,_xlpm.B_o,_xlpm.MMS_m,_xlpm.MCF_im,_xlpm.rho, _xlpm.VS_jkl * _xlpm.B_o * _xlpm.MMS_m * _xlpm.MCF_im * _xlpm.rho)</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__2_MethaneProductionFromManure_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(7, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VS_jkl","volatile solid production","kg/day","Calculated from 4.2.1.1 (3)";"B_o","emissions potential","m3 CH4/kg VS","Constant";"MMS_m","fraction of waste in each manure management system","fraction","Input";"MCF_im","methane conversion factor for temperature zone and MMS","fraction","Constant";"rho","density of methane","kg/m3","Constant";"i","state","","Input";"i","region","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__2_MethaneProductionFromManure_Arguments_Method2">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VS_jkl","volatile solid production","kg/day","Calculated from 4.2.1.1 (3)";"B_o","emissions potential","m3 CH4/kg VS","Constant";"MMS_m","fraction of waste in each manure management system","fraction","Input";"MCF_im","methane conversion factor for temperature zone and MMS","fraction","Constant";"rho","density of methane","kg/m3","Constant";"MAT","Mean annual temperature","°C","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__2_MethaneProductionFromManure_LatexEquation">_xlfn.LAMBDA("M_{jklm}=VS_{jkl}\times B_o\times MMS_m\times MCF_{im}\times \rho")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__2_MethaneProductionFromManure_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__2_MethaneProductionFromManure_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.1, Equation (2)")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__2_MethaneProductionFromManure_Title">_xlfn.LAMBDA("Methane production from the manure of grazing beef cattle")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__2_MethaneProductionFromManure_Unit">_xlfn.LAMBDA("kg CH4/head/day")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__2_MethaneProductionFromManure_Variable">_xlfn.LAMBDA("M_jklm")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__3_VolatileSolidProductionFromGrazingBeef">_xlfn.LAMBDA(_xlpm.I_jkl,_xlpm.DMD_jkl,_xlpm.A, (_xlpm.I_jkl * (1 - _xlpm.DMD_jkl) + (0.04 * _xlpm.I_jkl)) * (1 - _xlpm.A))</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__3_VolatileSolidProductionFromGrazingBeef_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"I_jkl","dry matter intake as calculated in Chapter 3 Section 3.2.1","kg/head/day","Calculated from 3.2.1.1, (3)";"DMD_jkl","dry matter digestibility expressed as a fraction","fraction","Input";"A","ash content of feed intake expressed as a fraction","fraction","Constant"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__3_VolatileSolidProductionFromGrazingBeef_LatexEquation">_xlfn.LAMBDA("VS_{jkl}=(I_{jkl}\times (1-DMD_{jkl})+(0.04\times I_{jkl}))\times (1-A)")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__3_VolatileSolidProductionFromGrazingBeef_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__3_VolatileSolidProductionFromGrazingBeef_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.1, Equation (3)")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__3_VolatileSolidProductionFromGrazingBeef_Title">_xlfn.LAMBDA("Volatile solid production from grazing beef")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__3_VolatileSolidProductionFromGrazingBeef_Unit">_xlfn.LAMBDA("kg/head/day")</definedName>
-    <definedName name="MMS_PastureBeef_Methane_Equations.VEERG_4_2_1_1__3_VolatileSolidProductionFromGrazingBeef_Variable">_xlfn.LAMBDA("VS_jkl")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture">_xlfn.LAMBDA(_xlpm.M_vol,_xlpm.EF_N2O,_xlpm.C_N2O, _xlpm.M_vol * _xlpm.EF_N2O * _xlpm.C_N2O * 10 ^ -3)</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"M_vol","mass of nitrogen volatilised from urine and faeces deposited on pasture","kg N","Calculated from 4.2.1.5 (2)";"EF_N2O","nitrous oxide emission factor for atmospheric deposition","kg N2O-N/kg N","Constant";"C_N2O","factor to convert elemental mass of N2O to molecular mass","","Constant";"j","production system","","Input";"i","irrigation method","","Input";"r","rainfall zone","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_LatexEquation">_xlfn.LAMBDA("E_{N2O,ad}=M_{vol}\times EF_{N2O}\times C_{N2O}\times 10^{-3}")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.5, Equation (1)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_Title">_xlfn.LAMBDA("Atmospheric deposition emissions from urine and dung deposited on pasture")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_Unit">_xlfn.LAMBDA("t N2O")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_Variable">_xlfn.LAMBDA("E_N2Oad")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__2_MassOfNitrogenVolatilisedOnPasture">_xlfn.LAMBDA(_xlpm.AE,_xlpm.FracGASMsoil, _xlpm.AE * _xlpm.FracGASMsoil)</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__2_MassOfNitrogenVolatilisedOnPasture_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"AE","total mass of nitrogen excreted on PRP for beef cattle","kg N","Calculated from 4.2.1.3 (2)";"FracGASMsoil","fraction of nitrogen volatilised from urine and faeces deposited on pasture ((kg NH3-N + NOx-N)/kg N)","fraction","Constant"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__2_MassOfNitrogenVolatilisedOnPasture_LatexEquation">_xlfn.LAMBDA("M_{vol}=AE\times FracGASMsoil")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__2_MassOfNitrogenVolatilisedOnPasture_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__2_MassOfNitrogenVolatilisedOnPasture_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.5, Equation (2)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__2_MassOfNitrogenVolatilisedOnPasture_Title">_xlfn.LAMBDA("Mass of nitrogen volatilised")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__2_MassOfNitrogenVolatilisedOnPasture_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_AtmosphericDeposition_Equations.VEERG_4_2_1_5__2_MassOfNitrogenVolatilisedOnPasture_Variable">_xlfn.LAMBDA("M_vol")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture">_xlfn.LAMBDA(_xlpm.M_leach,_xlpm.EF_leach,_xlpm.C_N2O, _xlpm.M_leach * _xlpm.EF_leach * _xlpm.C_N2O * 10 ^ -3)</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"M_leach","mass of nitrogen lost to leaching and runoff","kg N","Calculated from 4.2.1.7 (2)";"EF_leach","emission factor for leaching and runoff","kg N2O-N/kg N","Constant";"C_N2O","factor to convert elemental mass of N2O to molecular mass","","Constant"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_LatexEquation">_xlfn.LAMBDA("E_{N2O,leach}=M_{leach}\times EF_{leach}\times C_{N2O}\times 10^{-3}")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.7, Equation (1)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_Title">_xlfn.LAMBDA("Leaching and runoff emissions from urine and dung deposited on pasture")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_Unit">_xlfn.LAMBDA("t N2O")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_Variable">_xlfn.LAMBDA("E_N2Oleach")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__2_MassOfNitrogenLostToLeachingAndRunoffOnPasture">_xlfn.LAMBDA(_xlpm.AE,_xlpm.FracWet,_xlpm.FracLEACH, _xlpm.AE * _xlpm.FracWet * _xlpm.FracLEACH)</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__2_MassOfNitrogenLostToLeachingAndRunoffOnPasture_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"AE","total mass of nitrogen excreted on PRP for beef cattle","kg N","Calculated from 4.2.1.3 (2)";"FracWet","fraction of N available for leaching and runoff","fraction","Constant";"FracLEACH","fraction of all N that is lost through leaching and runoff","fraction","Constant";"z","location in leaching zone","","Input";"j","production system","","Input";"ir","irrigation method","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__2_MassOfNitrogenLostToLeachingAndRunoffOnPasture_LatexEquation">_xlfn.LAMBDA("M_{leach}=AE\times FracWet\times FracLEACH")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__2_MassOfNitrogenLostToLeachingAndRunoffOnPasture_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__2_MassOfNitrogenLostToLeachingAndRunoffOnPasture_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.7, Equation (2)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__2_MassOfNitrogenLostToLeachingAndRunoffOnPasture_Title">_xlfn.LAMBDA("Mass of nitrogen lost to leaching and runoff")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__2_MassOfNitrogenLostToLeachingAndRunoffOnPasture_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_LeachingAndRunoff.VEERG_4_2_1_7__2_MassOfNitrogenLostToLeachingAndRunoffOnPasture_Variable">_xlfn.LAMBDA("M_leach")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture">_xlfn.LAMBDA(_xlpm.AE,_xlpm.EF_PRP,_xlpm.C_N2O, _xlpm.AE * _xlpm.EF_PRP * _xlpm.C_N2O * 10 ^ -3)</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"AE","total mass of nitrogen excreted on PRP for beef cattle","kg N","Calculated from 4.2.1.3 (2)";"EF_PRP","emission factor for nitrous oxide from urine and dung deposited to soil","kg N2O-N/kg N deposited","Constant";"C_N2O","factor to convert elemental mass of nitrous oxide to molecular mass","","Constant";"z","wet or dry climate zone","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_LatexEquation">_xlfn.LAMBDA("E_{N2O,dir}=AE\times EF_{PRP}\times C_{N2O}\times 10^{-3}")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.3, Equation (1)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_Title">_xlfn.LAMBDA("Total annual direct nitrous oxide emissions from agricultural soils from deposition of urine and dung")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_Unit">_xlfn.LAMBDA("t N2O")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_Variable">_xlfn.LAMBDA("E_N2Odir")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__2_TotalNitrogenExcretedToPastureRangeAndPaddock">_xlfn.LAMBDA(_xlpm.N_jkl,_xlpm.NE_jkl,_xlpm.D_j, SUM((_xlpm.N_jkl * _xlpm.NE_jkl) * _xlpm.D_j))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__2_TotalNitrogenExcretedToPastureRangeAndPaddock_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"N_jkl","number of beef cattle by time-period, class and subclass","head","Input";"NE_jkl","nitrogen excreted in each time-period, by each class and subclass","kg N/head/day","Calculated from 4.2.1.3 (3)";"D_j","number of days in each time-period (days)","days","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__2_TotalNitrogenExcretedToPastureRangeAndPaddock_LatexEquation">_xlfn.LAMBDA("AE=\sum_{j}\sum_{k}\sum_{l}(N_{jkl}\times NE_{jkl}\times D_j)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__2_TotalNitrogenExcretedToPastureRangeAndPaddock_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__2_TotalNitrogenExcretedToPastureRangeAndPaddock_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.3, Equation (2)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__2_TotalNitrogenExcretedToPastureRangeAndPaddock_Title">_xlfn.LAMBDA("Total nitrogen excreted to pasture, range and paddock")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__2_TotalNitrogenExcretedToPastureRangeAndPaddock_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__2_TotalNitrogenExcretedToPastureRangeAndPaddock_Variable">_xlfn.LAMBDA("AE")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__3_NitrogenExcreted">_xlfn.LAMBDA(_xlpm.I_jkl,_xlpm.CP_j,_xlpm.MC_jk136,_xlpm.NR_jkl,_xlpm.W_jkl, ((_xlpm.I_jkl * _xlpm.CP_j) / 6.25) + ((0.032 * _xlpm.MC_jk136) / 6.38) - _xlpm.NR_jkl - ((1.1 * 10 ^ -4 * _xlpm.W_jkl ^ 0.75) / 6.25))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__3_NitrogenExcreted_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(7, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"I_jkl","dry matter intake as calculated in Chapter 3 Section 3.2.1 (kg DM/head/day)","kg DM/head/day","Calculated from 3.2.1.1 (3)";"CP_j","crude protein content of dry matter intake","fraction","Input";"MC_jk136","milk intake (kg/head/day)","kg/head/day","Constant";"NR_jkl","the amount of nitrogen retained by the body (kg N/head/day)","kg N/head/day","Calculated from 4.2.1.3 (4)";"W_jkl","liveweight (kg/head)","kg/head","Input";"b","breed of cattle","","Input";"s","Calving season","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__3_NitrogenExcreted_LatexEquation">_xlfn.LAMBDA("NE_{jkl}= (I_{jkl}\times CP_j \div 6.25)  + (0.032\times MC_{jk=1,3,6} \div 6.38)  - NR_{jkl} - \left[ (1.1\times 10^{-4}\times W_{jkl}^{0.75}) \div  6.25 \right]")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__3_NitrogenExcreted_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__3_NitrogenExcreted_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.3, Equation (3)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__3_NitrogenExcreted_Title">_xlfn.LAMBDA("Nitrogen excreted")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__3_NitrogenExcreted_Unit">_xlfn.LAMBDA("kg N/head/day")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__3_NitrogenExcreted_Variable">_xlfn.LAMBDA("NE_jkl")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__4_NitrogenRetainedByBody">_xlfn.LAMBDA(_xlpm.MP_jk5,_xlpm.L_jkl,_xlpm.Z_jkl,_xlpm.LWG_jkl, ((0.032 * _xlpm.MP_jk5) / 6.38) + (((0.212 - 0.008 * (_xlpm.L_jkl - 2) - ((0.14 - 0.008 * (_xlpm.L_jkl - 2)) / (1 + EXP(-6 * (_xlpm.Z_jkl - 0.4))))) * (_xlpm.LWG_jkl * 0.92)) / 6.25))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__4_NitrogenRetainedByBody_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"MP_jk5","milk production (kg/head/day)","kg/head/day","Calculated from 4.2.1.3 (5)";"L_jkl","intake relative to that needed for maintenance","","Calculated from 4.2.1.3 (6)";"Z_jkl","relative size","","Calculated from 4.2.1.3 (7)";"LWG_jkl","liveweight gain (kg/head/day)","kg/head/day","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__4_NitrogenRetainedByBody_LatexEquation">_xlfn.LAMBDA("NR_{jkl}=(0.032 \times MP_{jk=5} \div 6.38) + \left { \left { 0.212 - 0.008 \times (L_{jkl} -2) - \left[ \frac{0.140-0.008 \times (L_{jkl} - 2)}{1+e^{(-6 \times (Z_{jkl}-0.4))}} \right] \right} \times (LWG_{jkl} \times 0.92) \right} \div 6.25")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__4_NitrogenRetainedByBody_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__4_NitrogenRetainedByBody_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.3, Equation (4)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__4_NitrogenRetainedByBody_Title">_xlfn.LAMBDA("Amount of nitrogen retained by the body")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__4_NitrogenRetainedByBody_Unit">_xlfn.LAMBDA("kg N/head/day")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__4_NitrogenRetainedByBody_Variable">_xlfn.LAMBDA("NR_jkl")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason">_xlfn.LAMBDA(_xlpm.LC_jk5,_xlpm.DMP_jk5, _xlpm.LC_jk5 * _xlpm.DMP_jk5)</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"LC_jk5","proportion of cows greater than 2 years lactating for the season of calving and season after calving expressed as a fraction","fraction","Input";"DMP_jk5","daily milk production (kg/head/day)","kg/head/day","Constant";"b","breed of cattle","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason_ArgumentsVariation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(5, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"LC_jk5curr","proportion of cows greater than 2 years lactating for the season of calving","fraction","Input";"LC_jk5prev","proportion of cows greater than 2 years lactating for the season after calving","fraction","Input";"DMP_jk5calv","daily milk production for the season of calving (kg/head/day)","kg/head/day","Constant";"DMP_jk5after","daily milk production for the season after calving (kg/head/day)","kg/head/day","Constant";"b","breed of cattle","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason_LatexEquation">_xlfn.LAMBDA("MP_{jk=5}=LC_{jk=5}\times DMP_{jk=5}")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason_LatexEquationVariation">_xlfn.LAMBDA("MP_{jk=5}=(LC_{jk=5,current}\times DMP_{jk=5,calv})+(LC_{jk=5,prev}\times DMP_{jk=5,after})")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.3, Equation (5)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason_Title">_xlfn.LAMBDA("Milk production for the season of calving and season after calving")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason_Unit">_xlfn.LAMBDA("kg/head/day")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason_Variable">_xlfn.LAMBDA("MP_jk5")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeason_Variation">_xlfn.LAMBDA("VARIATION ON SOURCE: Split LC and DMP into calving season and after calving season values.")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__5_MilkProductionForCalvingSeasonVariation">_xlfn.LAMBDA(_xlpm.LC_jk5curr,_xlpm.LC_jk5prev,_xlpm.DMP_jk5calv,_xlpm.DMP_jk5after, (_xlpm.LC_jk5curr * _xlpm.DMP_jk5calv) + (_xlpm.LC_jk5prev * _xlpm.DMP_jk5after))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__6_IntakeRelativeToMaintenance">_xlfn.LAMBDA(_xlpm.I_jkl,_xlpm.W_jkl, _xlpm.I_jkl / ((1.185 + 0.00454 * _xlpm.W_jkl - 0.0000026 * _xlpm.W_jkl ^ 2) ^ 2))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__6_IntakeRelativeToMaintenance_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"I_jkl","dry matter intake as calculated in Chapter 3 Section 3.2.1 (kg DM/head/day)","kg DM/head/day","Calculated from 3.2.1.1 (3)";"W_jkl","liveweight (kg/head)","kg/head","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__6_IntakeRelativeToMaintenance_LatexEquation">_xlfn.LAMBDA("L_{jkl}=\frac{I_{jkl}}{(1.185+0.00454\times W_{jkl}-0.0000026\times W_{jkl}^{2})^{2}}")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__6_IntakeRelativeToMaintenance_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__6_IntakeRelativeToMaintenance_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.3, Equation (6)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__6_IntakeRelativeToMaintenance_Title">_xlfn.LAMBDA("Intake relative to that needed for maintenance")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__6_IntakeRelativeToMaintenance_Unit">_xlfn.LAMBDA("ratio")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__6_IntakeRelativeToMaintenance_Variable">_xlfn.LAMBDA("L_jkl")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__7_RelativeSize">_xlfn.LAMBDA(_xlpm.W_jkl,_xlpm.SRW_k, _xlpm.W_jkl / _xlpm.SRW_k)</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__7_RelativeSize_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"W_jkl","liveweight (kg)","kg","Input";"SRW_k","standard reference weight (kg)","kg","Constant";"i","state","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__7_RelativeSize_LatexEquation">_xlfn.LAMBDA("Z_{jkl}=\frac{W_{jkl}}{SRW_k}")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__7_RelativeSize_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__7_RelativeSize_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.1.3, Equation (7)")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__7_RelativeSize_Title">_xlfn.LAMBDA("Relative size of the cattle")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__7_RelativeSize_Unit">_xlfn.LAMBDA("ratio")</definedName>
-    <definedName name="MMS_PastureBeef_Soil_N2ODirect_Equations.VEERG_4_2_1_3__7_RelativeSize_Variable">_xlfn.LAMBDA("Z_jkl")</definedName>
-    <definedName name="Range_LivestockStartingValues">#REF!</definedName>
     <definedName name="Result_CarbonRemovalsFromPlantings">Results!$E$53</definedName>
     <definedName name="Result_EmissionsForWholeProductionCycle_Method1">Results!$E$42</definedName>
     <definedName name="Result_EmissionsForWholeProductionCycle_Method2">Results!$F$42</definedName>
@@ -424,92 +209,12 @@
     <definedName name="Result_Enterprise_Method2">Results!$I$28</definedName>
     <definedName name="Result_NetEmissions_Method1">Results!$E$59</definedName>
     <definedName name="Result_NetEmissions_Method2">Results!$F$59</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_AshContentOfFeedIntake_Data">_xlfn.LAMBDA(0.08)</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_AshContentOfFeedIntake_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.2.3 CONSTANTS")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_AshContentOfFeedIntake_Title">_xlfn.LAMBDA("Ash content of feed intake")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_AshContentOfFeedIntake_Unit">_xlfn.LAMBDA("fraction")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_AshContentOfFeedIntake_Variable">_xlfn.LAMBDA("A")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_AshContentOfFeedIntake_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_CrudeProteinContent_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(16, 6, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State","Region","Spring","Summer","Autumn","Winter";"ACT","n/a",0.07,0.13,0.1,0.06;"NSW","n/a",0.07,0.13,0.1,0.06;"NT","Alice Springs",0.058,0.092,0.075,0.053;"NT","Barkly",0.058,0.092,0.075,0.053;"NT","Northern",0.058,0.092,0.075,0.053;"QLD","High",0.072,0.099,0.078,0.059;"QLD","Moderate/High",0.072,0.099,0.078,0.059;"QLD","Moderate/Low",0.072,0.099,0.078,0.059;"QLD","Low",0.072,0.099,0.078,0.059;"SA","n/a",0.16,0.07,0.09,0.2;"TAS","n/a",0.2,0.1,0.16,0.2;"VIC","n/a",0.25,0.07,0.1,0.21;"WA","South West",0.2,0.09,0.06,0.2;"WA","Pilbara",0.04,0.12,0.09,0.06;"WA","Kimberley",0.04,0.12,0.09,0.06}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_CrudeProteinContent_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.2.6")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_CrudeProteinContent_Title">_xlfn.LAMBDA("Beef pasture cattle - Crude protein content of feed intake (fraction) (CPj)")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_CrudeProteinContent_Unit">_xlfn.LAMBDA("fraction")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_CrudeProteinContent_Variable">_xlfn.LAMBDA("CPj")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_CrudeProteinContent_Variation">_xlfn.LAMBDA("VARIATION ON SOURCE: Split ACT and NSW into separate rows. Duplicated QLD and NT rows with regions from table A.1.2.2 to aid lookup")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_DryMatterDigestibility_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(16, 6, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State","Region","Spring","Summer","Autumn","Winter";"ACT","n/a",0.55,0.65,0.6,0.5;"NSW","n/a",0.55,0.65,0.6,0.5;"NT","Alice Springs",0.55,0.61,0.57,0.54;"NT","Barkly",0.55,0.61,0.57,0.54;"NT","Northern",0.55,0.61,0.57,0.54;"QLD","High",0.53,0.57,0.55,0.51;"QLD","Moderate/High",0.53,0.57,0.55,0.51;"QLD","Moderate/Low",0.53,0.57,0.55,0.51;"QLD","Low",0.53,0.57,0.55,0.51;"SA","n/a",0.7,0.55,0.55,0.75;"TAS","n/a",0.75,0.6,0.7,0.75;"VIC","n/a",0.8,0.55,0.6,0.76;"WA","South West",0.8,0.58,0.5,0.75;"WA","Pilbara",0.4,0.65,0.55,0.45;"WA","Kimberley",0.4,0.65,0.55,0.45}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_DryMatterDigestibility_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.2.5")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_DryMatterDigestibility_Title">_xlfn.LAMBDA("Beef pasture cattle - Dry matter digestibility of feed intake (fraction) (DMDj)")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_DryMatterDigestibility_Unit">_xlfn.LAMBDA("fraction")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_DryMatterDigestibility_Variable">_xlfn.LAMBDA("DMDj")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_DryMatterDigestibility_Variation">_xlfn.LAMBDA("VARIATION ON SOURCE: Split ACT and NSW into separate rows. Duplicated QLD and NT rows with regions from table A.1.2.2 to aid lookup")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FeedAdjustmentAndMilkProduction_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Breed","Season","Feed adjustment (MCjk=1,3,6)","Milk intake / production (DMPjk=5)";"Hereford or Shorthorn breeds","Spring",1.3,6;"Hereford or Shorthorn breeds","Summer",1.1,4;"Hereford or Shorthorn breeds","Autumn",0,0;"Hereford or Shorthorn breeds","Winter",0,0;"Northern Brahman cross breed","Spring",0,0;"Northern Brahman cross breed","Summer",1.3,4;"Northern Brahman cross breed","Autumn",1.1,3;"Northern Brahman cross breed","Winter",0,0}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FeedAdjustmentAndMilkProduction_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.2.7")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FeedAdjustmentAndMilkProduction_Title">_xlfn.LAMBDA("Beef pasture cattle - Feed intake adjustment and milk production (kg/head/day)")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FeedAdjustmentAndMilkProduction_Unit">_xlfn.LAMBDA("")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FeedAdjustmentAndMilkProduction_Variable">_xlfn.LAMBDA("MCjk=1,3,6; DMPjk=5")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FeedAdjustmentAndMilkProduction_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracGASMSoil_Data">_xlfn.LAMBDA(0.21)</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracGASMSoil_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.2.3 CONSTANTS")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracGASMSoil_Title">_xlfn.LAMBDA("Fraction of nitrogen volatilised from urine and faeces deposited on pasture")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracGASMSoil_Unit">_xlfn.LAMBDA("fraction")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracGASMSoil_Variable">_xlfn.LAMBDA("FracGASMSoil")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracGASMSoil_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracLEACH_Data">_xlfn.LAMBDA(0.24)</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracLEACH_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.2.3 CONSTANTS")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracLEACH_Title">_xlfn.LAMBDA("Default fraction of N that is lost through leaching and runoff")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracLEACH_Unit">_xlfn.LAMBDA("fraction")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracLEACH_Variable">_xlfn.LAMBDA("FracLEACH")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FracLEACH_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FractionOfManureToMMS_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(16, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State","Region","Pasture range and paddock","Uncovered Anaerobic lagoon";"ACT","n/a",99.192,0.808;"NSW","n/a",99.452,0.548;"SA","n/a",99.759,0.241;"TAS","n/a",99.122,0.878;"VIC","n/a",98.894,1.106;"WA","South West",99.622,0.378;"WA","Pilbara",99.999,0.001;"WA","Kimberley",99.999,0.001;"NT","Alice Springs",99.999,0.001;"NT","Barkly",99.994,0.006;"NT","Northern",99.999,0.001;"QLD","High",99.773,0.227;"QLD","Moderate/High",99.898,0.102;"QLD","Moderate/Low",99.979,0.021;"QLD","Low",99.977,0.023}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FractionOfManureToMMS_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.2.9")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FractionOfManureToMMS_Title">_xlfn.LAMBDA("Beef pasture cattle - Fraction of manure to each manure management system (fraction) (MMSm)")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FractionOfManureToMMS_Unit">_xlfn.LAMBDA("fraction")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FractionOfManureToMMS_Variable">_xlfn.LAMBDA("MMSm")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_FractionOfManureToMMS_Variation">_xlfn.LAMBDA("VARIATION ON SOURCE: Removed comma from 'Pasture range and paddock' to aid lookup")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_Liveweight_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(29, 10, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State","Region","Season","Bull &lt; 1","Bull &gt; 1","Cow &lt; 1","Cow 1-2","Cow &gt; 2","Steer &lt; 1","Steer &gt; 1";"ACT/NSW","n/a","Spring",80,480,75,300,440,75,380;"ACT/NSW","n/a","Summer",170,520,160,360,470,160,420;"ACT/NSW","n/a","Autumn",240,550,220,390,490,220,450;"ACT/NSW","n/a","Winter",280,560,260,410,500,260,460;"South Australia","n/a","Spring",250,800,220,400,500,230,420;"South Australia","n/a","Summer",320,800,280,420,500,290,420;"South Australia","n/a","Autumn",80,700,70,300,450,75,400;"South Australia","n/a","Winter",160,700,140,350,450,150,400;"Tasmania","n/a","Spring",105,700,85,300,490,90,480;"Tasmania","n/a","Summer",480,750,150,350,530,160,460;"Tasmania","n/a","Autumn",250,725,200,360,500,215,490;"Tasmania","n/a","Winter",260,700,210,380,460,230,470;"Victoria","n/a","Spring",250,820,240,410,560,240,510;"Victoria","n/a","Summer",280,850,260,440,550,270,520;"Victoria","n/a","Autumn",100,700,95,300,450,95,410;"Victoria","n/a","Winter",150,720,140,320,470,140,440;"Western Australia","South West","Spring",340,800,260,420,550,300,480;"Western Australia","South West","Summer",380,780,300,450,530,340,470;"Western Australia","South West","Autumn",100,680,80,320,480,100,340;"Western Australia","South West","Winter",190,700,150,330,490,170,360;"Western Australia","Pilbara","Spring",80,450,70,260,340,80,370;"Western Australia","Pilbara","Summer",150,500,140,310,360,150,400;"Western Australia","Pilbara","Autumn",230,550,220,330,380,230,420;"Western Australia","Pilbara","Winter",250,500,240,340,360,250,390;"Western Australia","Kimberley","Spring",220,500,180,300,320,210,340;"Western Australia","Kimberley","Summer",110,550,90,220,380,100,390;"Western Australia","Kimberley","Autumn",170,600,140,270,390,160,430;"Western Australia","Kimberley","Winter",200,550,150,280,350,190,400}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_Liveweight_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.2.1")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_Liveweight_Title">_xlfn.LAMBDA("Beef pasture cattle - Liveweight (kg) (Wjkl)")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_Liveweight_Unit">_xlfn.LAMBDA("kg")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_Liveweight_Variable">_xlfn.LAMBDA("Wjkl")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_Liveweight_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGain_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(29, 10, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State","Region","Season","Bull &lt;1","Bull &gt;1","Cow &lt;1","Cow 1-2","Cow &gt;2","Steer &lt;1","Steer &gt;1";"ACT/NSW","n/a","Spring",0.5,0.2,0.5,0.4,0.3,0.5,0.4;"ACT/NSW","n/a","Summer",1,0.4,0.9,0.7,0.3,0.9,0.4;"ACT/NSW","n/a","Autumn",0.8,0.3,0.7,0.3,0.2,0.7,0.3;"ACT/NSW","n/a","Winter",0.4,0.1,0.4,0.2,0.1,0.4,0.1;"South Australia","n/a","Spring",0.99,1.1,0.88,0.55,0.55,0.88,0.22;"South Australia","n/a","Summer",0.77,0,0.66,0.22,0,0.66,0;"South Australia","n/a","Autumn",0.9,-1.1,0.7,0.22,-0.55,0.8,-0.22;"South Australia","n/a","Winter",0.88,0,0.77,0.55,0,0.82,0;"Tasmania","n/a","Spring",1,0.5,1,1,-0.44,1,0.5;"Tasmania","n/a","Summer",0.82,0.55,0.71,0.55,0.99,0.77,0.5;"Tasmania","n/a","Autumn",0.77,0.5,0.55,0.11,-0.33,0.6,0.33;"Tasmania","n/a","Winter",0.11,-0.27,0.11,0.22,-0.44,0.16,-0.22;"Victoria","n/a","Spring",1.1,1.1,1.1,0.99,0.99,1.1,0.77;"Victoria","n/a","Summer",0.33,0.33,0.22,0.33,-0.1,0.33,0.11;"Victoria","n/a","Autumn",0.5,0.2,0.55,0.44,0.2,0.55,0.2;"Victoria","n/a","Winter",0.55,0.22,0.49,0.22,0.22,0.49,0.33;"Western Australia","South West","Spring",1.64,1.1,1.21,0.99,0.66,1.42,1.1;"Western Australia","South West","Summer",0.44,-0.22,0.44,0.33,-0.22,0.44,-0.11;"Western Australia","South West","Autumn",0.6,0,0.6,0.22,-0.55,0.6,0;"Western Australia","South West","Winter",0.99,0.22,0.77,0.11,0.11,0.77,0.44;"Western Australia","Pilbara","Spring",0.7,-0.55,0.7,0.22,-0.22,0.7,-0.22;"Western Australia","Pilbara","Summer",0.77,0.55,0.77,0.66,0.55,0.77,0.33;"Western Australia","Pilbara","Autumn",0.88,0.55,0.88,0.22,0.22,0.88,0.22;"Western Australia","Pilbara","Winter",0.22,-0.55,0.22,0.11,-0.22,0.22,-0.33;"Western Australia","Kimberley","Spring",0.22,-0.55,0.33,0.22,-0.33,0.22,-0.55;"Western Australia","Kimberley","Summer",0.8,0.55,0.7,0.44,0.66,0.8,0.55;"Western Australia","Kimberley","Autumn",0.66,0.55,0.55,0.55,0.11,0.66,0.55;"Western Australia","Kimberley","Winter",0.33,-0.55,0.11,0.11,-0.44,0.33,-0.55}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGain_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.2.3")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGain_Title">_xlfn.LAMBDA("Beef pasture cattle - Liveweight gain (kg) (LWGjkl)")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGain_Unit">_xlfn.LAMBDA("kg")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGain_Variable">_xlfn.LAMBDA("LWGjkl")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGain_Variation">_xlfn.LAMBDA("VARIATION ON SOURCE: Replaced 'n/a' with 'South West' for first four rows of Western Australia to be consistent with table A.1.2.1")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGainNTQLD_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(29, 13, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State","Region","Season","Bull &lt;1","Bull &gt;1","Cow &lt;1","Cow 1-2","Cow 2-3","Cow &gt;3","Steer &lt;1","Steer 1-2","Steer 2-3","Steer &gt;3";"Northern Territory","Alice Springs","Spring",0.22,-0.23,0.25,0.17,0.18,-0.28,0.32,0.24,0.25,-0.05;"Northern Territory","Alice Springs","Summer",0.66,0.2,0.62,0.54,0.38,0.27,0.75,0.64,0.55,0.48;"Northern Territory","Alice Springs","Autumn",0.49,0.13,0.54,0.45,0.35,0.15,0.63,0.54,0.42,0.26;"Northern Territory","Alice Springs","Winter",0.27,-0.8,0.22,0.09,0.12,0.02,0.25,0.18,0.12,0.03;"Northern Territory","Barkly","Spring",0.22,-0.44,0.2,0.21,0.18,0.01,0.12,0.09,"NO","NO";"Northern Territory","Barkly","Summer",0.66,0.22,0.68,0.22,0.24,0.25,0.64,0.37,"NO","NO";"Northern Territory","Barkly","Autumn",0.49,0.05,0.64,0.25,0.29,0.12,0.57,0.49,"NO","NO";"Northern Territory","Barkly","Winter",0.27,-0.27,0.31,0.29,0.19,0.04,0.26,0.28,"NO","NO";"Northern Territory","Northern","Spring",0.22,-0.44,0,0.15,0.08,0.17,0.06,0.02,-0.14,"NO";"Northern Territory","Northern","Summer",0.66,0.22,0.79,0.4,0.38,0.27,0.8,0.16,0.3,"NO";"Northern Territory","Northern","Autumn",0.49,0.05,0.55,0.38,0.36,0.06,0.58,0.23,0.4,"NO";"Northern Territory","Northern","Winter",0.27,-0.27,0.02,0.09,0.16,-0.04,0.21,0.03,0.11,"NO";"Queensland","High","Spring",0.27,-0.19,0.38,0.25,0.07,0.05,0.52,0.55,0.19,0.6;"Queensland","High","Summer",0.16,0.16,0.8,0.57,0.76,0.49,0.84,0.51,0.36,0.17;"Queensland","High","Autumn",0.45,0.1,0.49,0.41,0.4,0.17,0.54,0.64,-0.05,0.32;"Queensland","High","Winter",0.51,-0.07,0.13,-0.09,-0.13,0.07,0.25,0.71,0.17,0.43;"Queensland","Moderate/High","Spring",-0.12,-0.19,0.41,0.09,0.41,-0.19,0.07,1.07,-0.08,0;"Queensland","Moderate/High","Summer",0.65,0.19,0.65,0.51,0.18,0.63,1.3,0.48,1.12,0.38;"Queensland","Moderate/High","Autumn",0.7,0.13,0.52,0.34,0.02,0.04,0.77,0.42,0.12,0.74;"Queensland","Moderate/High","Winter",0.32,-0.06,0.25,0.19,-0.1,-0.02,0.02,0.23,-0.13,0;"Queensland","Moderate/Low","Spring",0.62,-0.19,0.37,0.41,0.06,-0.02,0.47,0.44,0.3,0.13;"Queensland","Moderate/Low","Summer",0.05,0.19,0.31,0.54,0.53,0.15,0.28,0.57,0.42,0.4;"Queensland","Moderate/Low","Autumn",0.33,0.13,0.39,0.36,0.26,0.11,0.4,0.44,0.37,-0.01;"Queensland","Moderate/Low","Winter",0.61,-0.06,0.21,0.18,0.12,0.06,0.29,0.41,0.41,-0.15;"Queensland","Low","Spring",-0.2,0.02,0.24,0.3,0.23,-0.05,0.34,0.3,0.57,0.52;"Queensland","Low","Summer",0.62,0.21,0.25,0.32,0.47,0.31,0.14,0.4,0.26,0.43;"Queensland","Low","Autumn",0.4,0.13,0.12,0.27,0.3,0.08,0.13,0.24,0.15,0.21;"Queensland","Low","Winter",0.08,0.04,0.06,0.18,0.11,-0.07,0.13,0.16,0.4,0.33}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGainNTQLD_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.2.4")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGainNTQLD_Title">_xlfn.LAMBDA("Beef pasture cattle - Liveweight gain (kg) (LWGjkl) for NT and QLD")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGainNTQLD_Unit">_xlfn.LAMBDA("kg")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGainNTQLD_Variable">_xlfn.LAMBDA("LWGjkl")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightGainNTQLD_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightNTQLD_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(29, 13, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State","Region","Season","Bull &lt;1","Bull &gt;1","Cows &lt;1","Cows 1-2","Cows 2-3","Cows &gt;3","Steer &lt;1","Steer 1-2","Steer 2-3","Steer &gt;3";"Northern Territory","Alice Springs","Spring",220,706,208,323,415,467,223,371,493,585;"Northern Territory","Alice Springs","Summer",110,703,112,256,368,465,108,280,421,543;"Northern Territory","Alice Springs","Autumn",170,721,169,306,392,464,176,339,470,580;"Northern Territory","Alice Springs","Winter",200,727,211,338,432,492,222,377,498,590;"Northern Territory","Barkly","Spring",220,620,227,319,398,452,216,334,"NO","NO";"Northern Territory","Barkly","Summer",110,650,108,262,346,430,111,236,"NO","NO";"Northern Territory","Barkly","Autumn",170,670,170,266,363,444,169,282,"NO","NO";"Northern Territory","Barkly","Winter",200,660,225,307,398,452,214,326,"NO","NO";"Northern Territory","Northern","Spring",220,620,177,267,365,406,231,249,324,"NO";"Northern Territory","Northern","Summer",110,650,102,203,299,380,102,218,263,"NO";"Northern Territory","Northern","Autumn",170,670,173,250,336,414,175,243,304,"NO";"Northern Territory","Northern","Winter",200,660,202,272,365,390,208,260,337,"NO";"Queensland","High","Spring",260,705,215,302,416,519,234,455,551,660;"Queensland","High","Summer",153,703,118,277,397,483,111,304,521,547;"Queensland","High","Autumn",168,718,191,319,440,506,188,326,520,582;"Queensland","High","Winter",235,722,207,352,470,514,209,421,512,605;"Queensland","Moderate/High","Spring",230,674,217,344,357,467,242,370,550,620;"Queensland","Moderate/High","Summer",113,669,113,283,361,477,120,273,545,553;"Queensland","Moderate/High","Autumn",172,685,172,309,376,471,238,329,573,620;"Queensland","Moderate/High","Winter",241,692,208,344,364,484,260,350,567,620;"Queensland","Moderate/Low","Spring",236,674,178,310,428,466,193,370,519,565;"Queensland","Moderate/Low","Summer",120,669,112,250,390,448,115,273,433,556;"Queensland","Moderate/Low","Autumn",125,685,140,277,407,455,141,296,445,593;"Queensland","Moderate/Low","Winter",180,692,183,316,438,468,189,354,500,553;"Queensland","Low","Spring",190,617,174,265,371,415,170,272,392,531;"Queensland","Low","Summer",119,591,140,205,310,405,133,218,315,445;"Queensland","Low","Autumn",175,610,163,232,351,427,146,242,320,471;"Queensland","Low","Winter",192,615,162,255,364,420,157,261,342,484}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightNTQLD_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.2.2")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightNTQLD_Title">_xlfn.LAMBDA("Beef pasture cattle - Liveweight (kg) (Wjkl) for NT and QLD")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightNTQLD_Unit">_xlfn.LAMBDA("kg")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightNTQLD_Variable">_xlfn.LAMBDA("Wjkl")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_LiveweightNTQLD_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneConversionFactorPerRegion_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(16, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State","Region","Pasture range and paddock","Uncovered Anaerobic lagoon";"ACT","n/a",0.0047,0.71;"NSW","n/a",0.0047,0.75;"SA","n/a",0.0047,0.74;"TAS","n/a",0.0047,0.7;"VIC","n/a",0.0047,0.74;"WA","South West",0.0047,0.76;"WA","Pilbara",0.0047,0.76;"WA","Kimberley",0.0047,0.76;"NT","Alice Springs",0.0047,0.8;"NT","Barkly",0.0047,0.8;"NT","Northern",0.0047,0.8;"QLD","High",0.0047,0.78;"QLD","Moderate/High",0.0047,0.78;"QLD","Moderate/Low",0.0047,0.78;"QLD","Low",0.0047,0.78}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneConversionFactorPerRegion_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.2.10")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneConversionFactorPerRegion_Title">_xlfn.LAMBDA("Beef pasture cattle - Methane conversion factor per region (fraction) (MCFim)")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneConversionFactorPerRegion_Unit">_xlfn.LAMBDA("fraction")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneConversionFactorPerRegion_Variable">_xlfn.LAMBDA("MCFim")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneConversionFactorPerRegion_Variation">_xlfn.LAMBDA("VARIATION ON SOURCE: Removed comma from 'Pasture range and paddock' to aid lookup")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneEmissionsPotential_Data">_xlfn.LAMBDA(0.19)</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneEmissionsPotential_Source">_xlfn.LAMBDA("VEERG 2026: 4.2.2.3 CONSTANTS")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneEmissionsPotential_Title">_xlfn.LAMBDA("Methane emissions potential")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneEmissionsPotential_Unit">_xlfn.LAMBDA("m3 CH4 / kg VS")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneEmissionsPotential_Variable">_xlfn.LAMBDA("B0")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_MethaneEmissionsPotential_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_StandardReferenceWeights_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 9, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State","Bulls &lt;1","Bulls &gt;1","Cows &lt;1","Cows 1-2","Cows &gt;2","Steer &lt;1","Steer &gt;1","State abbreviation";"ACT",700,700,500,500,500,600,600,"ACT";"NSW",700,700,500,500,500,600,600,"NSW";"Northern Territory",770,770,550,550,550,660,660,"NT";"Queensland",770,770,550,550,550,660,660,"QLD";"South Australia",770,770,550,550,550,660,660,"SA";"Tasmania",770,770,550,550,550,660,660,"TAS";"Victoria",770,770,550,550,550,660,660,"VIC";"Western Australia",770,770,550,550,550,660,660,"WA"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_StandardReferenceWeights_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.2.8")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_StandardReferenceWeights_Title">_xlfn.LAMBDA("Beef pasture cattle - Standard reference weights (kg) (SRWk)")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_StandardReferenceWeights_Unit">_xlfn.LAMBDA("kg")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_StandardReferenceWeights_Variable">_xlfn.LAMBDA("SRWk")</definedName>
-    <definedName name="SourceData_PastureBeef.SourceData_PastureBeef_StandardReferenceWeights_Variation">_xlfn.LAMBDA("VARIATION ON SOURCE: Split ACT and NSW into separate rows. Added 'State abbreviation' column to aid lookup.")</definedName>
     <definedName name="X_Cell_Enterprise_ProductionTimeframeEnd">'Input - Enterprise'!$E$19</definedName>
     <definedName name="X_Cell_Enterprise_ProductionTimeframeStart">'Input - Enterprise'!$E$18</definedName>
+    <definedName name="X_Cell_Fertiliser_AreaUnderCropping">'Input - Fert Prod System'!$E$10</definedName>
+    <definedName name="X_Cell_Fertiliser_CropType">'Input - Fert Prod System'!$E$8</definedName>
+    <definedName name="X_Cell_Fertiliser_IrrigationMethod">'Input - Fert Prod System'!$E$9</definedName>
+    <definedName name="X_Cell_Fertiliser_ProductionSystem">'Input - Fert Prod System'!$E$7</definedName>
     <definedName name="X_Cell_Site_AverageTemperature">'Input - Site'!$E$14</definedName>
     <definedName name="X_Cell_Site_ClimateZone">'Input - Site'!$E$20</definedName>
     <definedName name="X_Cell_Site_Elevation">'Input - Site'!$E$13</definedName>
@@ -587,7 +292,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="199">
   <si>
     <t>Home</t>
   </si>
@@ -626,9 +331,6 @@
   </si>
   <si>
     <t>CO2-e emissions method 2</t>
-  </si>
-  <si>
-    <t>4.2 Manure management: Pasture Beef: Results</t>
   </si>
   <si>
     <t>4.2.1.1-2 Manure methane</t>
@@ -1045,12 +747,6 @@
     <t>Unit</t>
   </si>
   <si>
-    <t>Emissions allocation (mass)</t>
-  </si>
-  <si>
-    <t>Manure sold</t>
-  </si>
-  <si>
     <t>t co2e/t liveweight sold</t>
   </si>
   <si>
@@ -1168,9 +864,6 @@
     <t>14.1.1-2 Purchased electricity (Market-based)</t>
   </si>
   <si>
-    <t>Enter value</t>
-  </si>
-  <si>
     <t>Input - Enterprise</t>
   </si>
   <si>
@@ -1202,6 +895,54 @@
   </si>
   <si>
     <t>=SUM(Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells('Input - Pasture Beef'!X_Table_PastureBeef_Head_Method1, 'Input - Pasture Beef'!X_Table_PastureBeef_Duration_Method1, '4.2.1.1-2 Methane'!M1_Table_VS_j_k_l))*10^-3</t>
+  </si>
+  <si>
+    <t>Product emissions - Mass</t>
+  </si>
+  <si>
+    <t>Product emissions - Economic</t>
+  </si>
+  <si>
+    <t>Mass emissions assignment</t>
+  </si>
+  <si>
+    <t>Economic emissions assignment</t>
+  </si>
+  <si>
+    <t>Emissions per tonne liveweight grown</t>
+  </si>
+  <si>
+    <t>Liveweight sold - excluding removals</t>
+  </si>
+  <si>
+    <t>Liveweight sold - net emissions</t>
+  </si>
+  <si>
+    <t>Manure sold - excluding removals</t>
+  </si>
+  <si>
+    <t>Manure sold - net emissions</t>
+  </si>
+  <si>
+    <t>Enterprise: Pasture Beef: Results</t>
+  </si>
+  <si>
+    <t>Input - Fertiliser Production System</t>
+  </si>
+  <si>
+    <t>Production system</t>
+  </si>
+  <si>
+    <t>Crop type</t>
+  </si>
+  <si>
+    <t>Area under cropping</t>
+  </si>
+  <si>
+    <t>Pasture</t>
+  </si>
+  <si>
+    <t>These inputs are used for fertiliser calculations, and they take their values from the "Input - Pasture" sheet. Do not edit these cells.</t>
   </si>
 </sst>
 </file>
@@ -2044,7 +1785,7 @@
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="4" borderId="0" xfId="8">
       <alignment horizontal="left" vertical="center"/>
@@ -2290,6 +2031,9 @@
     <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="25" fillId="4" borderId="2" xfId="52" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="0" xfId="47">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="69">
@@ -3472,745 +3216,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:doughnutChart>
-        <c:varyColors val="1"/>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:showLeaderLines val="0"/>
-        </c:dLbls>
-        <c:firstSliceAng val="0"/>
-        <c:holeSize val="75"/>
-      </c:doughnutChart>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:noFill/>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:noFill/>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050">
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="25400">
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>938212</xdr:colOff>
-      <xdr:row>65</xdr:row>
-      <xdr:rowOff>200025</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1443037</xdr:colOff>
-      <xdr:row>77</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Chart 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0DEA1AD2-453E-4F97-8BC2-DE4AF27985BA}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks/>
-        </xdr:cNvGraphicFramePr>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
 <rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>
@@ -5022,7 +4027,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>13</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -5107,7 +4112,7 @@
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E7" s="19" t="e" cm="1">
         <f t="array" ref="E7">VEERG_3_2_1_1__1_TotalAnnualMethaneFromEntericFermentation_Result_Method1</f>
@@ -5140,7 +4145,7 @@
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" s="19" t="e" cm="1">
         <f t="array" ref="E8">VEERG_4_2_1_1__1_TotalAnnualMethaneProductionFromManureManagement_Result_Method1</f>
@@ -5170,7 +4175,7 @@
       <c r="A9" s="5"/>
       <c r="C9" s="9"/>
       <c r="D9" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E9" s="19" t="e" cm="1">
         <f t="array" ref="E9">VEERG_4_2_1_3__1_DirectNitrousOxideEmissionsOnPasture_Result_Method1</f>
@@ -5181,7 +4186,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H9" s="19" t="e" cm="1">
         <f t="array" ref="H9">Common_Equations.Common_ConvertN2OToCO2e(E9,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5202,7 +4207,7 @@
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E10" s="19" t="e" cm="1">
         <f t="array" ref="E10">VEERG_4_2_1_5__1_AtmosphericDepositionEmissionsFromUrineAndDungOnPasture_Result_Method1</f>
@@ -5213,7 +4218,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H10" s="19" t="e" cm="1">
         <f t="array" ref="H10">Common_Equations.Common_ConvertN2OToCO2e(E10,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5235,7 +4240,7 @@
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E11" s="19" t="e" cm="1">
         <f t="array" ref="E11">VEERG_4_2_1_7__1_LeachingAndRunoffEmissionsFromUrineAndDungOnPasture_Result_Method1</f>
@@ -5246,7 +4251,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H11" s="19" t="e" cm="1">
         <f t="array" ref="H11">Common_Equations.Common_ConvertN2OToCO2e(E11,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5268,7 +4273,7 @@
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E12" s="19" t="e" cm="1">
         <f t="array" ref="E12">VEERG_5_1_1_1__1_InorganicFertiliserApplicationN2OEmissions_Result_Method1</f>
@@ -5279,7 +4284,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H12" s="19" t="e" cm="1">
         <f t="array" ref="H12">Common_Equations.Common_ConvertN2OToCO2e(E12,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5301,7 +4306,7 @@
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E13" s="19" t="e" cm="1">
         <f t="array" ref="E13">VEERG_5_1_1_3__1_InorganicFertiliserApplicationCO2Emissions_Result_Method1</f>
@@ -5312,7 +4317,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H13" s="19" t="e">
         <f>E13</f>
@@ -5334,7 +4339,7 @@
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E14" s="19" t="e" cm="1">
         <f t="array" ref="E14">VEERG_5_2_1_1__2_MassOfNitrogenInOrganicFertiliser_Result_Method1</f>
@@ -5345,7 +4350,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H14" s="19" t="e" cm="1">
         <f t="array" ref="H14">Common_Equations.Common_ConvertN2OToCO2e(E14,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5364,7 +4369,7 @@
       <c r="A15" s="5"/>
       <c r="C15" s="9"/>
       <c r="D15" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E15" s="19" t="e" cm="1">
         <f t="array" ref="E15">VEERG_5_3_1_1__1_LimeApplicationCO2Emissions_Result_Method1</f>
@@ -5375,7 +4380,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H15" s="19" t="e">
         <f>E15</f>
@@ -5396,7 +4401,7 @@
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E16" s="19" t="e" cm="1">
         <f t="array" ref="E16">VEERG_5_4_1_3__1_OrganicFertiliserAtmosphericDepositionN2OEmissions_Result_Method1</f>
@@ -5407,7 +4412,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H16" s="19" t="e" cm="1">
         <f t="array" ref="H16">Common_Equations.Common_ConvertN2OToCO2e(E16,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5429,7 +4434,7 @@
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="1" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E17" s="19" t="e" cm="1">
         <f t="array" ref="E17">VEERG_5_5_1_1__1_FertiliserLeachingAndRunoffN2OEmissions_result_Method1</f>
@@ -5440,7 +4445,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H17" s="19" t="e" cm="1">
         <f t="array" ref="H17">Common_Equations.Common_ConvertN2OToCO2e(E17,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5462,7 +4467,7 @@
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="E18" s="19" t="e" cm="1">
         <f t="array" ref="E18">VEERG_6_2_1_1__1__NitrousOxideEmissionsFromPastureResidues_Result_Method1</f>
@@ -5473,7 +4478,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H18" s="19" t="e" cm="1">
         <f t="array" ref="H18">Common_Equations.Common_ConvertN2OToCO2e(E18,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5495,7 +4500,7 @@
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="1" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E19" s="19" t="e" cm="1">
         <f t="array" ref="E19">VEERG_6_3_1_1__1__LeachingAndRunoffEmissionsCropAndPastureResidue_PastureOnly_Result_Method1</f>
@@ -5506,7 +4511,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H19" s="19" t="e" cm="1">
         <f t="array" ref="H19">Common_Equations.Common_ConvertN2OToCO2e(E19,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5528,7 +4533,7 @@
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="1" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E20" s="19" t="e" cm="1">
         <f t="array" ref="E20">VEERG_8_1_1_1__1_FuelCombustionTransport_Result_CO2</f>
@@ -5539,7 +4544,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H20" s="19" t="e">
         <f>E20</f>
@@ -5557,7 +4562,7 @@
     <row r="21" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="9"/>
       <c r="D21" s="1" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E21" s="19" t="e" cm="1">
         <f t="array" ref="E21">VEERG_8_1_1_1__1_FuelCombustionTransport_Result_CH4</f>
@@ -5587,7 +4592,7 @@
       <c r="A22" s="5"/>
       <c r="C22" s="9"/>
       <c r="D22" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E22" s="19" t="e" cm="1">
         <f t="array" ref="E22">VEERG_8_1_1_1__1_FuelCombustionTransport_Result_N2O</f>
@@ -5598,7 +4603,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H22" s="19" t="e" cm="1">
         <f t="array" ref="H22">Common_Equations.Common_ConvertN2OToCO2e(E22,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5617,7 +4622,7 @@
       <c r="A23" s="5"/>
       <c r="C23" s="9"/>
       <c r="D23" s="1" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E23" s="19" t="e" cm="1">
         <f t="array" ref="E23">VEERG_8_2_1_1__1_FuelCombustionStationary_Result_CO2</f>
@@ -5628,7 +4633,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H23" s="19" t="e">
         <f>E23</f>
@@ -5647,7 +4652,7 @@
       <c r="A24" s="5"/>
       <c r="C24" s="9"/>
       <c r="D24" s="1" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E24" s="19" t="e" cm="1">
         <f t="array" ref="E24">VEERG_8_2_1_1__1_FuelCombustionStationary_Result_CH4</f>
@@ -5676,7 +4681,7 @@
     <row r="25" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="9"/>
       <c r="D25" s="1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E25" s="19" t="e" cm="1">
         <f t="array" ref="E25">VEERG_8_2_1_1__1_FuelCombustionStationary_Result_N2O</f>
@@ -5687,7 +4692,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H25" s="19" t="e" cm="1">
         <f t="array" ref="H25">Common_Equations.Common_ConvertN2OToCO2e(E25,_xlfn.XLOOKUP("N2O", Table_GWPData[Gas],Table_GWPData[CO2-e factor]))</f>
@@ -5705,7 +4710,7 @@
     <row r="26" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="9"/>
       <c r="D26" s="1" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E26" s="19" t="e" cm="1">
         <f t="array" ref="E26">VEERG_14_1_1__1_LocationBasedScopeElectricityEmissions_Result_Method1</f>
@@ -5734,7 +4739,7 @@
     <row r="27" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="9"/>
       <c r="D27" s="1" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E27" s="19" t="e" cm="1">
         <f t="array" ref="E27">VEERG_14_1_2__1_MarketBasedScopeElectricityEmissionsVariation_Result_Method1</f>
@@ -5817,7 +4822,7 @@
     <row r="32" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C32" s="9"/>
       <c r="D32" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
@@ -5844,7 +4849,7 @@
     <row r="34" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C34" s="9"/>
       <c r="D34" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -5868,7 +4873,7 @@
     <row r="36" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C36" s="9"/>
       <c r="D36" s="21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E36" s="21" t="s">
         <v>11</v>
@@ -5987,7 +4992,7 @@
     <row r="42" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C42" s="9"/>
       <c r="D42" s="15" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E42" s="20" t="e">
         <f>SUM(E37:E41)</f>
@@ -6028,7 +5033,7 @@
     <row r="45" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C45" s="9"/>
       <c r="D45" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -6052,10 +5057,10 @@
     <row r="47" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C47" s="9"/>
       <c r="D47" s="21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
@@ -6070,11 +5075,12 @@
         <f t="array" ref="D48:D50">Common_InputFunctions.getOverlappingReportingPeriods(X_Cell_Enterprise_ProductionTimeframeStart,X_Cell_Enterprise_ProductionTimeframeEnd,X_Cell_Site_StartDate)</f>
         <v>01 Jan 2023 to 31 Dec 2023</v>
       </c>
-      <c r="E48" s="87">
-        <v>0.6</v>
+      <c r="E48" s="87" t="str">
+        <f>IF(ISBLANK(D48), "", "Enter value")</f>
+        <v>Enter value</v>
       </c>
       <c r="F48" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
@@ -6087,11 +5093,12 @@
       <c r="D49" s="1" t="str">
         <v>01 Jan 2024 to 31 Dec 2024 (This reporting cycle)</v>
       </c>
-      <c r="E49" s="87">
-        <v>0.5</v>
+      <c r="E49" s="87" t="str">
+        <f t="shared" ref="E49:E52" si="1">IF(ISBLANK(D49), "", "Enter value")</f>
+        <v>Enter value</v>
       </c>
       <c r="F49" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
@@ -6104,11 +5111,12 @@
       <c r="D50" s="1" t="str">
         <v>01 Jan 2025 to 31 Dec 2025</v>
       </c>
-      <c r="E50" s="87" t="s">
-        <v>175</v>
+      <c r="E50" s="87" t="str">
+        <f t="shared" si="1"/>
+        <v>Enter value</v>
       </c>
       <c r="F50" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
@@ -6119,9 +5127,12 @@
     <row r="51" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C51" s="9"/>
       <c r="D51" s="1"/>
-      <c r="E51" s="87"/>
+      <c r="E51" s="87" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F51" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
@@ -6132,9 +5143,12 @@
     <row r="52" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C52" s="9"/>
       <c r="D52" s="1"/>
-      <c r="E52" s="87"/>
+      <c r="E52" s="87" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F52" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
@@ -6145,11 +5159,11 @@
     <row r="53" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C53" s="9"/>
       <c r="D53" s="15" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E53" s="20">
         <f>SUM(E48:E51)</f>
-        <v>1.1000000000000001</v>
+        <v>0</v>
       </c>
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
@@ -6183,7 +5197,7 @@
     <row r="56" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C56" s="9"/>
       <c r="D56" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
@@ -6208,10 +5222,10 @@
       <c r="C58" s="9"/>
       <c r="D58" s="21"/>
       <c r="E58" s="21" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="F58" s="21" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
@@ -6222,7 +5236,7 @@
     <row r="59" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C59" s="9"/>
       <c r="D59" s="90" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E59" s="88" t="e">
         <f>E42-E53</f>
@@ -6251,273 +5265,380 @@
     </row>
     <row r="61" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C61" s="9"/>
-      <c r="D61" s="21" t="s">
-        <v>156</v>
-      </c>
-      <c r="E61" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="F61" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="G61" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="H61" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="I61" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="J61" s="21" t="s">
-        <v>133</v>
-      </c>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
+      <c r="H61" s="1"/>
+      <c r="I61" s="1"/>
+      <c r="J61" s="1"/>
       <c r="K61" s="9"/>
     </row>
     <row r="62" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C62" s="9"/>
-      <c r="D62" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="F62" s="19" t="str">
-        <f>'Input - Enterprise'!E22</f>
-        <v>=SUM(Table_Input_LivestockSales[Total liveweight sold])*10^-3</v>
-      </c>
-      <c r="G62" s="19" t="e">
-        <f>F62/(F62+F63)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H62" s="19" t="e">
-        <f>($E$42/F62)*G62</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="I62" s="19" t="e">
-        <f>($F$42/F62)*G62</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="J62" s="16" t="s">
-        <v>136</v>
-      </c>
+      <c r="D62" s="92" t="s">
+        <v>183</v>
+      </c>
+      <c r="E62" s="1"/>
+      <c r="F62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="H62" s="1"/>
+      <c r="I62" s="1"/>
+      <c r="J62" s="1"/>
       <c r="K62" s="9"/>
     </row>
     <row r="63" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C63" s="9"/>
-      <c r="D63" s="1" t="s">
+      <c r="D63" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="E63" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="F63" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="G63" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="H63" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="E63" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F63" s="19" t="e">
-        <f>'Input - Enterprise'!E25*'Input - Enterprise'!E26</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G63" s="19" t="e">
-        <f>F63/(F62+F63)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H63" s="19" t="e">
-        <f>($E$42/F63)*G63</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="I63" s="19" t="e">
-        <f>($F$42/F63)*G63</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="J63" s="16" t="s">
-        <v>137</v>
+      <c r="I63" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="J63" s="21" t="s">
+        <v>132</v>
       </c>
       <c r="K63" s="9"/>
     </row>
     <row r="64" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C64" s="9"/>
       <c r="D64" s="1" t="s">
-        <v>143</v>
+        <v>188</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="F64" s="19" t="e">
-        <f>'Input - Enterprise'!E25*'Input - Enterprise'!E27</f>
+        <v>138</v>
+      </c>
+      <c r="F64" s="19" t="str">
+        <f>'Input - Enterprise'!E22</f>
+        <v>=SUM(Table_Input_LivestockSales[Total liveweight sold])*10^-3</v>
+      </c>
+      <c r="G64" s="19" t="e">
+        <f>F64/(F64+F66)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G64" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="H64" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="I64" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="J64" s="9"/>
+      <c r="H64" s="19" t="e">
+        <f>(Result_EmissionsForWholeProductionCycle_Method1/F64)*G64</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I64" s="19" t="e">
+        <f>(Result_EmissionsForWholeProductionCycle_Method2/F64)*G64</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J64" s="16" t="s">
+        <v>133</v>
+      </c>
       <c r="K64" s="9"/>
     </row>
     <row r="65" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C65" s="9"/>
-      <c r="D65" s="1"/>
-      <c r="E65" s="1"/>
-      <c r="F65" s="19"/>
-      <c r="G65" s="19"/>
-      <c r="H65" s="19"/>
-      <c r="I65" s="19"/>
-      <c r="J65" s="18"/>
+      <c r="D65" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F65" s="19" t="str">
+        <f>F64</f>
+        <v>=SUM(Table_Input_LivestockSales[Total liveweight sold])*10^-3</v>
+      </c>
+      <c r="G65" s="19" t="e">
+        <f>G64</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H65" s="19" t="e">
+        <f>(Result_NetEmissions_Method1/F65)*G65</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I65" s="19" t="e">
+        <f>(Result_NetEmissions_Method2/F65)*G65</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J65" s="16" t="s">
+        <v>133</v>
+      </c>
       <c r="K65" s="9"/>
     </row>
     <row r="66" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C66" s="9"/>
       <c r="D66" s="1" t="s">
-        <v>154</v>
+        <v>190</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="F66" s="19" t="str">
-        <f>'Input - Enterprise'!E23</f>
-        <v>=SUM(Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells('Input - Pasture Beef'!X_Table_PastureBeef_Head_Method1, 'Input - Pasture Beef'!X_Table_PastureBeef_Duration_Method1, 'Input - Pasture Beef'!X_Table_PastureBeef_LiveweightGain_Method1))*10^-3</v>
-      </c>
-      <c r="G66" s="19" t="s">
-        <v>144</v>
+        <v>139</v>
+      </c>
+      <c r="F66" s="19" t="e">
+        <f>'Input - Enterprise'!E25*'Input - Enterprise'!E26</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G66" s="19" t="e">
+        <f>F66/(F64+F66)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="H66" s="19" t="e">
-        <f>E59/F66</f>
+        <f>(Result_EmissionsForWholeProductionCycle_Method1/F66)*G66</f>
         <v>#NAME?</v>
       </c>
-      <c r="I66" s="19" t="s">
-        <v>144</v>
+      <c r="I66" s="19" t="e">
+        <f>(Result_EmissionsForWholeProductionCycle_Method2/F66)*G66</f>
+        <v>#NAME?</v>
       </c>
       <c r="J66" s="16" t="s">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="K66" s="9"/>
     </row>
     <row r="67" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C67" s="9"/>
       <c r="D67" s="1" t="s">
-        <v>155</v>
+        <v>191</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="F67" s="19" t="str">
-        <f>'Input - Enterprise'!E24</f>
-        <v>=SUM(Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells('Input - Pasture Beef'!X_Table_PastureBeef_Head_Method2, 'Input - Pasture Beef'!X_Table_PastureBeef_Duration_Method2, 'Input - Pasture Beef'!X_Table_PastureBeef_LiveweightGain_Method2))*10^-3</v>
-      </c>
-      <c r="G67" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="H67" s="19" t="s">
-        <v>144</v>
+        <v>139</v>
+      </c>
+      <c r="F67" s="19" t="e">
+        <f>F66</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G67" s="19" t="e">
+        <f>G66</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H67" s="19" t="e">
+        <f>(Result_NetEmissions_Method1/F67)*G67</f>
+        <v>#NAME?</v>
       </c>
       <c r="I67" s="19" t="e">
-        <f>F59/F67</f>
+        <f>(Result_NetEmissions_Method2/F67)*G67</f>
         <v>#NAME?</v>
       </c>
       <c r="J67" s="16" t="s">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="K67" s="9"/>
     </row>
     <row r="68" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C68" s="9"/>
-      <c r="D68" s="1"/>
-      <c r="E68" s="1"/>
-      <c r="F68" s="1"/>
-      <c r="G68" s="1"/>
-      <c r="H68" s="18"/>
-      <c r="I68" s="18"/>
-      <c r="J68" s="18"/>
+      <c r="D68" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F68" s="19" t="e">
+        <f>'Input - Enterprise'!E25*'Input - Enterprise'!E27</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G68" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="H68" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="I68" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="J68" s="9"/>
       <c r="K68" s="9"/>
     </row>
     <row r="69" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C69" s="9"/>
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
-      <c r="F69" s="1"/>
-      <c r="G69" s="1"/>
-      <c r="H69" s="9"/>
-      <c r="I69" s="9"/>
-      <c r="J69" s="9"/>
+      <c r="F69" s="19"/>
+      <c r="G69" s="19"/>
+      <c r="H69" s="19"/>
+      <c r="I69" s="19"/>
+      <c r="J69" s="18"/>
       <c r="K69" s="9"/>
     </row>
     <row r="70" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C70" s="9"/>
-      <c r="D70" s="1"/>
+      <c r="D70" s="92" t="s">
+        <v>184</v>
+      </c>
       <c r="E70" s="1"/>
       <c r="F70" s="1"/>
       <c r="G70" s="1"/>
-      <c r="H70" s="9"/>
-      <c r="I70" s="9"/>
-      <c r="J70" s="9"/>
+      <c r="H70" s="1"/>
+      <c r="I70" s="1"/>
+      <c r="J70" s="1"/>
       <c r="K70" s="9"/>
     </row>
     <row r="71" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C71" s="9"/>
-      <c r="D71" s="1"/>
-      <c r="E71" s="1"/>
-      <c r="F71" s="1"/>
-      <c r="G71" s="1"/>
-      <c r="H71" s="9"/>
-      <c r="I71" s="9"/>
-      <c r="J71" s="9"/>
+      <c r="D71" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="E71" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="F71" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="G71" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="H71" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="I71" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="J71" s="21" t="s">
+        <v>132</v>
+      </c>
       <c r="K71" s="9"/>
     </row>
     <row r="72" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C72" s="9"/>
-      <c r="D72" s="1"/>
-      <c r="E72" s="1"/>
-      <c r="F72" s="1"/>
-      <c r="G72" s="1"/>
-      <c r="H72" s="9"/>
-      <c r="I72" s="9"/>
-      <c r="J72" s="9"/>
+      <c r="D72" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F72" s="19" t="str">
+        <f>F64</f>
+        <v>=SUM(Table_Input_LivestockSales[Total liveweight sold])*10^-3</v>
+      </c>
+      <c r="G72" s="19">
+        <f>'Input - Enterprise'!E31</f>
+        <v>0.8</v>
+      </c>
+      <c r="H72" s="19" t="e">
+        <f>(Result_EmissionsForWholeProductionCycle_Method1/F72)*G72</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I72" s="19" t="e">
+        <f>(Result_EmissionsForWholeProductionCycle_Method2/F72)*G72</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J72" s="16" t="s">
+        <v>133</v>
+      </c>
       <c r="K72" s="9"/>
     </row>
     <row r="73" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C73" s="9"/>
-      <c r="D73" s="1"/>
-      <c r="E73" s="1"/>
-      <c r="F73" s="1"/>
-      <c r="G73" s="1"/>
-      <c r="H73" s="1"/>
-      <c r="I73" s="1"/>
-      <c r="J73" s="1"/>
+      <c r="D73" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F73" s="19" t="str">
+        <f>F64</f>
+        <v>=SUM(Table_Input_LivestockSales[Total liveweight sold])*10^-3</v>
+      </c>
+      <c r="G73" s="19">
+        <f>G72</f>
+        <v>0.8</v>
+      </c>
+      <c r="H73" s="19" t="e">
+        <f>(Result_NetEmissions_Method1/F73)*G73</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I73" s="19" t="e">
+        <f>(Result_NetEmissions_Method2/F73)*G73</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J73" s="16" t="s">
+        <v>133</v>
+      </c>
       <c r="K73" s="9"/>
     </row>
     <row r="74" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C74" s="9"/>
-      <c r="D74" s="1"/>
-      <c r="E74" s="1"/>
-      <c r="F74" s="1"/>
-      <c r="G74" s="1"/>
-      <c r="H74" s="1"/>
-      <c r="I74" s="1"/>
-      <c r="J74" s="1"/>
+      <c r="D74" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F74" s="19" t="e">
+        <f>F66</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G74" s="19">
+        <f>'Input - Enterprise'!E32</f>
+        <v>0.2</v>
+      </c>
+      <c r="H74" s="19" t="e">
+        <f>(Result_EmissionsForWholeProductionCycle_Method1/F74)*G74</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I74" s="19" t="e">
+        <f>(Result_EmissionsForWholeProductionCycle_Method2/F74)*G74</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J74" s="16" t="s">
+        <v>134</v>
+      </c>
       <c r="K74" s="9"/>
     </row>
     <row r="75" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C75" s="9"/>
-      <c r="D75" s="1"/>
-      <c r="E75" s="1"/>
-      <c r="F75" s="1"/>
-      <c r="G75" s="1"/>
-      <c r="H75" s="1"/>
-      <c r="I75" s="1"/>
-      <c r="J75" s="1"/>
+      <c r="D75" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F75" s="19" t="e">
+        <f>F67</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G75" s="19">
+        <f>G74</f>
+        <v>0.2</v>
+      </c>
+      <c r="H75" s="19" t="e">
+        <f>(Result_NetEmissions_Method1/F75)*G75</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I75" s="19" t="e">
+        <f>(Result_NetEmissions_Method2/F75)*G75</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J75" s="16" t="s">
+        <v>134</v>
+      </c>
       <c r="K75" s="9"/>
     </row>
     <row r="76" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C76" s="9"/>
-      <c r="D76" s="1"/>
-      <c r="E76" s="1"/>
-      <c r="F76" s="1"/>
-      <c r="G76" s="1"/>
-      <c r="H76" s="1"/>
-      <c r="I76" s="1"/>
-      <c r="J76" s="1"/>
+      <c r="D76" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F76" s="19" t="e">
+        <f>F68</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G76" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="H76" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="I76" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="J76" s="9"/>
       <c r="K76" s="9"/>
     </row>
     <row r="77" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -6531,9 +5652,11 @@
       <c r="J77" s="1"/>
       <c r="K77" s="9"/>
     </row>
-    <row r="78" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="3:11" ht="18.75" x14ac:dyDescent="0.25">
       <c r="C78" s="9"/>
-      <c r="D78" s="1"/>
+      <c r="D78" s="92" t="s">
+        <v>187</v>
+      </c>
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
@@ -6544,35 +5667,81 @@
     </row>
     <row r="79" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C79" s="9"/>
-      <c r="D79" s="1"/>
-      <c r="E79" s="1"/>
-      <c r="F79" s="1"/>
-      <c r="G79" s="1"/>
-      <c r="H79" s="1"/>
-      <c r="I79" s="1"/>
-      <c r="J79" s="1"/>
+      <c r="D79" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="E79" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="F79" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="G79" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="H79" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="I79" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="J79" s="21" t="s">
+        <v>132</v>
+      </c>
       <c r="K79" s="9"/>
     </row>
     <row r="80" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C80" s="9"/>
-      <c r="D80" s="1"/>
-      <c r="E80" s="1"/>
-      <c r="F80" s="1"/>
-      <c r="G80" s="1"/>
-      <c r="H80" s="1"/>
-      <c r="I80" s="1"/>
-      <c r="J80" s="1"/>
+      <c r="D80" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="F80" s="19" t="str">
+        <f>'Input - Enterprise'!E23</f>
+        <v>=SUM(Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells('Input - Pasture Beef'!X_Table_PastureBeef_Head_Method1, 'Input - Pasture Beef'!X_Table_PastureBeef_Duration_Method1, 'Input - Pasture Beef'!X_Table_PastureBeef_LiveweightGain_Method1))*10^-3</v>
+      </c>
+      <c r="G80" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="H80" s="19" t="e">
+        <f>E59/F80</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I80" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="J80" s="16" t="s">
+        <v>154</v>
+      </c>
       <c r="K80" s="9"/>
     </row>
     <row r="81" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C81" s="9"/>
-      <c r="D81" s="1"/>
-      <c r="E81" s="1"/>
-      <c r="F81" s="1"/>
-      <c r="G81" s="1"/>
-      <c r="H81" s="1"/>
-      <c r="I81" s="1"/>
-      <c r="J81" s="1"/>
+      <c r="D81" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="F81" s="19" t="str">
+        <f>'Input - Enterprise'!E24</f>
+        <v>=SUM(Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells('Input - Pasture Beef'!X_Table_PastureBeef_Head_Method2, 'Input - Pasture Beef'!X_Table_PastureBeef_Duration_Method2, 'Input - Pasture Beef'!X_Table_PastureBeef_LiveweightGain_Method2))*10^-3</v>
+      </c>
+      <c r="G81" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="H81" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="I81" s="19" t="e">
+        <f>F59/F81</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J81" s="16" t="s">
+        <v>154</v>
+      </c>
       <c r="K81" s="9"/>
     </row>
     <row r="82" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -6644,7 +5813,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -6672,7 +5840,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="39" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:24" s="33" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6730,7 +5898,7 @@
     </row>
     <row r="5" spans="1:24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D5" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="N5" s="42"/>
     </row>
@@ -6746,7 +5914,7 @@
         <v>Site</v>
       </c>
       <c r="D7" s="54" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E7" s="55"/>
       <c r="F7" s="55"/>
@@ -6758,7 +5926,7 @@
         <v>Pasture Beef</v>
       </c>
       <c r="D8" s="57" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E8" s="58"/>
       <c r="F8" s="58"/>
@@ -6776,13 +5944,13 @@
         <v>3</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="F10" s="27" t="s">
         <v>111</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>112</v>
       </c>
       <c r="N10" s="46"/>
     </row>
@@ -6792,13 +5960,13 @@
         <v>4.2.1.1-2 Methane</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E11" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="E11" s="24" t="s">
-        <v>114</v>
-      </c>
       <c r="F11" s="27" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G11" s="1"/>
       <c r="N11" s="51"/>
@@ -6809,13 +5977,13 @@
         <v>4.2.1.3-4 Soil direct N2O</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E12" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="E12" s="24" t="s">
-        <v>116</v>
-      </c>
       <c r="F12" s="27" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6824,13 +5992,13 @@
         <v>4.2.1.5-6 Soil atm. deposition</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E13" s="45">
         <v>307.7</v>
       </c>
       <c r="F13" s="27" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="N13" s="53"/>
       <c r="O13" s="53"/>
@@ -6841,13 +6009,13 @@
         <v>4.2.1.7-8 Soil leach &amp; runoff</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E14" s="45">
         <v>18</v>
       </c>
       <c r="F14" s="27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N14" s="53"/>
       <c r="O14" s="53"/>
@@ -6855,13 +6023,13 @@
     <row r="15" spans="1:24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="D15" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E15" s="45">
         <v>601</v>
       </c>
       <c r="F15" s="27" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="N15" s="53"/>
       <c r="O15" s="53"/>
@@ -6871,13 +6039,13 @@
         <v>2</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E16" s="45">
         <v>1326</v>
       </c>
       <c r="F16" s="27" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="N16" s="53"/>
       <c r="O16" s="53"/>
@@ -6888,13 +6056,13 @@
         <v>Constants - Pasture Beef</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E17" s="45">
         <v>7</v>
       </c>
       <c r="F17" s="27" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:25" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6903,7 +6071,7 @@
         <v>Constants - Livestock</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E18" s="26">
         <f>E15/E16</f>
@@ -6917,7 +6085,7 @@
         <v>Constants - Common</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E19" s="26" t="str">
         <f>Common_InputFunctions.Utility_LookupItemFromMinMax(E15,Table_SourceData_RainfallZones[Min rainfall],Table_SourceData_RainfallZones[Max rainfall],Table_SourceData_RainfallZones[Rainfall Zone])</f>
@@ -6932,7 +6100,7 @@
         <v>Acknowledgements</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E20" s="26" t="str">
         <f>Common_InputFunctions.Utility_GetClimateZone(E14,E15,E17,E13,E18,Table_SourceData_ClimateZones[Min temp],Table_SourceData_ClimateZones[Max temp],Table_SourceData_ClimateZones[Min rainfall],Table_SourceData_ClimateZones[Max rainfall],Table_SourceData_ClimateZones[Min frost days],Table_SourceData_ClimateZones[Max frost days],Table_SourceData_ClimateZones[Min elevation],Table_SourceData_ClimateZones[Max elevation],Table_SourceData_ClimateZones[Min MAP:PET],Table_SourceData_ClimateZones[Max MAP:PET],Table_SourceData_ClimateZones[Climate zone])</f>
@@ -6945,7 +6113,7 @@
     <row r="21" spans="1:25" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21"/>
       <c r="D21" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E21" s="26" t="str">
         <f>Common_InputFunctions.Utility_LookupValueInTable($E$20,Table_SourceData_WetDryZones[Climate zone],Table_SourceData_WetDryZones[Wet or Dry Zone])</f>
@@ -6957,7 +6125,7 @@
     <row r="22" spans="1:25" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="D22" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E22" s="26" t="str">
         <f>Common_InputFunctions.Utility_LookupItemFromMinMax(E14,Table_SourceData_TemperatureZones[Min MAT],Table_SourceData_TemperatureZones[Max MAT],Table_SourceData_TemperatureZones[Temperature Zone])</f>
@@ -7435,7 +6603,7 @@
   <sheetData>
     <row r="1" spans="3:10" ht="25.5" x14ac:dyDescent="0.35">
       <c r="C1" s="39" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D1" s="33"/>
       <c r="E1" s="33"/>
@@ -7467,7 +6635,7 @@
     </row>
     <row r="5" spans="3:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D5" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E5" s="36"/>
       <c r="F5" s="36"/>
@@ -7481,20 +6649,20 @@
     </row>
     <row r="7" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D7" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="45" t="s">
         <v>100</v>
-      </c>
-      <c r="E7" s="45" t="s">
-        <v>101</v>
       </c>
       <c r="F7" s="27"/>
       <c r="G7" s="36"/>
     </row>
     <row r="8" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D8" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="E8" s="45" t="s">
         <v>102</v>
-      </c>
-      <c r="E8" s="45" t="s">
-        <v>103</v>
       </c>
       <c r="F8" s="36"/>
       <c r="G8" s="36"/>
@@ -7507,7 +6675,7 @@
     </row>
     <row r="10" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D10" s="47" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E10" s="48"/>
       <c r="F10" s="49"/>
@@ -7521,26 +6689,26 @@
     </row>
     <row r="12" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D12" s="23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E12" s="25">
         <v>45292</v>
       </c>
       <c r="F12" s="27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G12" s="36"/>
     </row>
     <row r="13" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D13" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E13" s="52">
         <f>DATE(YEAR(E12)+1,MONTH(E12),DAY(E12))-1</f>
         <v>45657</v>
       </c>
       <c r="F13" s="27" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G13" s="36"/>
     </row>
@@ -7550,152 +6718,152 @@
     </row>
     <row r="16" spans="3:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D16" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D18" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E18" s="25">
         <v>45231</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D19" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E19" s="25">
         <v>45747</v>
       </c>
       <c r="F19" s="27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D20" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E20" s="26">
         <f>DATEDIF(E18,E19+1,"m")</f>
         <v>17</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="22" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D22" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E22" s="91" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="G22" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D23" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E23" s="91" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="G23" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D24" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E24" s="91" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="G24" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D25" s="1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E25" s="91" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="G25" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D26" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E26" s="91" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="G26" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D27" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E27" s="29">
         <v>0.1</v>
       </c>
       <c r="G27" s="27" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="28" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D28" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E28" s="29">
         <v>0.2</v>
       </c>
       <c r="G28" s="27" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="29" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D29" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E29" s="30">
         <f>100%-E27-E28</f>
         <v>0.7</v>
       </c>
       <c r="G29" s="27" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="31" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D31" s="1" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E31" s="29">
         <v>0.8</v>
       </c>
       <c r="G31" s="27" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="32" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D32" s="1" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E32" s="29">
         <v>0.2</v>
       </c>
       <c r="G32" s="27" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -7704,6 +6872,90 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7ECDB01-675B-437E-9BE1-C7A5D3E87BF1}">
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" style="1" customWidth="1"/>
+    <col min="4" max="10" width="30.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="17" customFormat="1" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="17" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D5" s="81" t="s">
+        <v>198</v>
+      </c>
+      <c r="E5" s="81"/>
+      <c r="F5" s="81"/>
+      <c r="G5" s="81"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F6" s="27"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D7" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="F7" s="27"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D8" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="F8" s="27"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D9" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="26" t="e" cm="1">
+        <f t="array" ref="E9">X_Cell_Pasture_IrrigationMethod</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D10" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="E10" s="26" t="e" cm="1">
+        <f t="array" ref="E10">X_Cell_Pasture_AreaUnderPasture</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD7772F5-D62F-448B-BE59-D05AA2138B09}">
   <dimension ref="A1:BY259"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -7736,7 +6988,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:65" s="3" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -7779,13 +7031,13 @@
     <row r="6" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6"/>
       <c r="D6" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="31" t="s">
+      <c r="F6" s="31" t="s">
         <v>34</v>
-      </c>
-      <c r="F6" s="31" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -7936,7 +7188,7 @@
     <row r="20" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20"/>
       <c r="D20" s="31" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8035,10 +7287,10 @@
     <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36"/>
       <c r="D36" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="E36" s="31" t="s">
         <v>37</v>
-      </c>
-      <c r="E36" s="31" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8131,19 +7383,19 @@
     </row>
     <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D47" s="31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E47" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="F47" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="F47" s="31" t="s">
+      <c r="G47" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="G47" s="31" t="s">
+      <c r="H47" s="31" t="s">
         <v>41</v>
-      </c>
-      <c r="H47" s="31" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8333,10 +7585,10 @@
     <row r="62" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="63" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D63" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="E63" s="31" t="s">
         <v>43</v>
-      </c>
-      <c r="E63" s="31" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="64" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8523,52 +7775,52 @@
     <row r="88" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="89" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D89" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E89" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="F89" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="F89" s="31" t="s">
+      <c r="G89" s="31" t="s">
         <v>46</v>
       </c>
-      <c r="G89" s="31" t="s">
+      <c r="H89" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="H89" s="31" t="s">
+      <c r="I89" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="I89" s="31" t="s">
+      <c r="J89" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="J89" s="31" t="s">
+      <c r="K89" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="K89" s="31" t="s">
+      <c r="L89" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="L89" s="31" t="s">
+      <c r="M89" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="M89" s="31" t="s">
+      <c r="N89" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="N89" s="31" t="s">
+      <c r="O89" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="O89" s="31" t="s">
+      <c r="P89" s="31" t="s">
         <v>55</v>
       </c>
-      <c r="P89" s="31" t="s">
+      <c r="Q89" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="Q89" s="31" t="s">
+      <c r="R89" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="R89" s="31" t="s">
+      <c r="S89" s="31" t="s">
         <v>58</v>
-      </c>
-      <c r="S89" s="31" t="s">
-        <v>59</v>
       </c>
       <c r="T89" s="31"/>
     </row>
@@ -9155,16 +8407,16 @@
     <row r="108" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="109" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D109" s="31" t="s">
+        <v>59</v>
+      </c>
+      <c r="E109" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="F109" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="E109" s="31" t="s">
-        <v>45</v>
-      </c>
-      <c r="F109" s="31" t="s">
+      <c r="G109" s="31" t="s">
         <v>61</v>
-      </c>
-      <c r="G109" s="31" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="110" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -9249,16 +8501,16 @@
     </row>
     <row r="119" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D119" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="E119" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="E119" s="31" t="s">
-        <v>64</v>
-      </c>
       <c r="F119" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="G119" s="31" t="s">
         <v>52</v>
-      </c>
-      <c r="G119" s="31" t="s">
-        <v>53</v>
       </c>
       <c r="BN119" s="33"/>
     </row>
@@ -9319,10 +8571,10 @@
     <row r="126" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="127" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D127" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="E127" s="31" t="s">
         <v>65</v>
-      </c>
-      <c r="E127" s="31" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="128" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -9363,10 +8615,10 @@
     </row>
     <row r="134" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D134" t="s">
+        <v>66</v>
+      </c>
+      <c r="E134" t="s">
         <v>67</v>
-      </c>
-      <c r="E134" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="135" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -9449,10 +8701,10 @@
     </row>
     <row r="142" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D142" s="31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E142" s="31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="BN142" s="33"/>
     </row>
@@ -9536,10 +8788,10 @@
     </row>
     <row r="153" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D153" s="31" t="s">
+        <v>69</v>
+      </c>
+      <c r="E153" s="31" t="s">
         <v>70</v>
-      </c>
-      <c r="E153" s="31" t="s">
-        <v>71</v>
       </c>
       <c r="BC153" s="36"/>
       <c r="BD153" s="36"/>
@@ -9809,19 +9061,19 @@
     </row>
     <row r="186" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D186" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="E186" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="E186" s="31" t="s">
+      <c r="F186" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="F186" s="31" t="s">
+      <c r="G186" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="G186" s="31" t="s">
+      <c r="H186" s="31" t="s">
         <v>75</v>
-      </c>
-      <c r="H186" s="31" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="187" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -10136,10 +9388,10 @@
     </row>
     <row r="206" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D206" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E206" s="31" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="207" spans="4:8" x14ac:dyDescent="0.25">
@@ -10170,10 +9422,10 @@
     </row>
     <row r="212" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D212" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="E212" s="31" t="s">
         <v>78</v>
-      </c>
-      <c r="E212" s="31" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="213" spans="4:5" x14ac:dyDescent="0.25">
@@ -10316,52 +9568,52 @@
     </row>
     <row r="231" spans="4:19" x14ac:dyDescent="0.25">
       <c r="D231" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="E231" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="E231" s="31" t="s">
+      <c r="F231" s="38" t="s">
         <v>81</v>
       </c>
-      <c r="F231" s="38" t="s">
+      <c r="G231" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="G231" s="31" t="s">
+      <c r="H231" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="H231" s="31" t="s">
+      <c r="I231" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="I231" s="31" t="s">
+      <c r="J231" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="J231" s="31" t="s">
+      <c r="K231" s="31" t="s">
         <v>86</v>
       </c>
-      <c r="K231" s="31" t="s">
+      <c r="L231" s="31" t="s">
         <v>87</v>
       </c>
-      <c r="L231" s="31" t="s">
+      <c r="M231" s="31" t="s">
         <v>88</v>
       </c>
-      <c r="M231" s="31" t="s">
+      <c r="N231" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="N231" s="31" t="s">
+      <c r="O231" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="O231" s="31" t="s">
+      <c r="P231" s="31" t="s">
         <v>91</v>
       </c>
-      <c r="P231" s="31" t="s">
+      <c r="Q231" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="Q231" s="31" t="s">
+      <c r="R231" s="31" t="s">
         <v>93</v>
       </c>
-      <c r="R231" s="31" t="s">
+      <c r="S231" s="31" t="s">
         <v>94</v>
-      </c>
-      <c r="S231" s="31" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="232" spans="4:19" x14ac:dyDescent="0.25">
@@ -11644,10 +10896,10 @@
     </row>
     <row r="257" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D257" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="E257" s="31" t="s">
         <v>96</v>
-      </c>
-      <c r="E257" s="31" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="258" spans="4:5" x14ac:dyDescent="0.25">
@@ -11696,6 +10948,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -11890,11 +11153,11 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBvAHcAcwAsAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgACYAIABcACIAIAB0AG8AIABcACIAIAAmACAAZQBuAGQAcwBUAGUAeAB0ACAAJgAgAHQAYQBnACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBvAHcAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAA+ADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjACcAXAAiACAAJgAgAHMAaAAgACYAIABcACIAJwAhAFwAIgAgACYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgACYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADEALAAgADIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADMALAAgADQAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAATQBNAFMALAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFwAbgAgACAAIAAgACAAIAAgACAATQBFAEQASQBBAE4AKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgACYAIABcACIAIABcACIAIAAmACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAIABkAGEAdABhACAAdABoAGEAdAAgAGkAcwAgAGMAbwBtAG0AbwBuACAAYQBjAHIAbwBzAHMAIABhAGwAbAAgAGUAbgB0AGUAcgBwAHIAaQBzAGUAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQA6ACAATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXABuAE4ASQBSAF8AMgAwADIAMwBfAFYAbwBsADEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAFwAbgBwACAAPQAgAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlACAAKAAwAC4ANgA3ADgANAAgAGsAZwAvAG0AMwApAFwAbgBUAGEAawBlAG4AIABmAHIAbwBtACAAdABoAGUAIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAYQBuAGQAIABFAG4AZQByAGcAeQAgAFIAZQBwAG8AcgB0AGkAbgBnACAAXABuACgATQBlAGEAcwB1AHIAZQBtAGUAbgB0ACkAIABEAGUAdABlAHIAbQBpAG4AYQB0AGkAbwBuACAAMgAwADAAOABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwACAAPQAgAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AbQAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AcwAgADMALgBCAC4AMQBhAF8AMgAsACAAMwAuAEIALgAxAGMAXwAyACwAIAAzAC4AQgAuADMAXwAxACwAIAAzAC4AQgAuADQAZwBfADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgA2ADcAOAA0ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBcAG4AQwBnACAAPQAgADQANAAvADIAOAAgAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBnAE4AMgBPAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQANAAvADIAOAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBcAG4ARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAGEAcwBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMQBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAyAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgAFwAIgAxADYALwAxADIAXAAiACwAIAAxADYALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgAFwAIgA0ADQALwAyADgAXAAiACwAIAA0ADQALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AeABcACIALAAgAFwAIgA0ADYALwAxADQAXAAiACwAIAA0ADYALAAgADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AXAAiACwAIABcACIAMgA4AC8AMQAyAFwAIgAsACAAMgA4ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAIABMAGkAbQBlAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ATQBWAE8AQwBcACIALAAgAFwAIgAxADQALwAxADIAXAAiACwAIAAxADQALAAgADEAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAATgAyAE8AXABuAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAVwBQAE4AMgBPAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAGEAcwBcACIALAAgAFwAIgBDAE8AMgAtAGUAIABmAGEAYwB0AG8AcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAMgA2ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBGADQAXAAiACwAIAA2ADYAMwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAMgBGADYAXAAiACwAIAAxADIAMgAwADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBGADYAXAAiACwAIAAyADIAOAAwADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBGADMAXAAiACwAIAAxADcAMgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAdABhAHQAZQBzACAAYQBuAGQAIAB0AGUAcgByAGkAdABvAHIAaQBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlAC8AVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQwBvAG0AbQBvAG4AIABOAGEAbQBlAFwAIgAsACAAXAAiAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEMAYQBwAGkAdABhAGwAIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBBAEMAVABcACIALAAgAFwAIgBBAEMAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAQQBTAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBOAFQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAQgBTACAAUwB0AGEAdABpAHMAdABjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADQAIAAtACAAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABCAHUAcgBlAGEAdQAgAG8AZgAgAFMAdABhAHQAaQBzAHQAaQBjAHMAIAAoAEEAQgBTACkAIAAtACAAUwB0AGEAdABpAHMAdABpAGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAAMgAgAC0AIAAyADAAMgAxACAALQAgAFMAaABhAHAAZQBmAGkAbABlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAxACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEEAIAA0ACAATgBhAG0AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AG4AYgB1AHIAeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAG4AZAB1AHIAYQBoAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAASQBuAG4AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAFcAaABlAGEAdAAgAEIAZQBsAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABOAG8AcgB0AGgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAFMAbwB1AHQAaAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHcAZQB0ACAAYQBuAGQAIABkAHIAeQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMgA6ACAAVAByAGEAbgBzAGwAYQB0AGkAbgBnACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwAgAHQAbwAgAHcAZQB0ACAAYQBuAGQAIABkAHIAeQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAC0AIABDAGgAYQBuAGcAZQBkACAAJwBGAHIAeQAnACAAdABvACAAJwBEAHIAeQAnAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAD4AIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgADEAMAAwADAALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAD4AIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAPgAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAPgAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADAAIABDACAALQAgAGQiIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAPgAgADYAMAAwAG0AbQBcACIALAAgADYAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZCIgADYAMAAwAG0AbQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADYAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAWgBvAG4AZQBcACIALAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABjAHIAaQB0AGUAcgBpAGEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAG8AYwBjAHUAcgBzAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQA+AKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIAAnAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQAnACAAcgBvAHcALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGEAcwB0AGUAcgBpAHMAawBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAAnAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAJwAsACAAJwByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACcAIABhAG4AZAAgACcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkACcAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHUAcABsAGkAYwBhAHQAZQBkACAAJwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQAnACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgACcAQQByAGUAYQBzACAAYQByAGUAIABzAHUAYgBqAGUAYwB0ACAAdABvACAAbABlAGEAYwBoAGkAbgBnACAAKABpAC4AZQAuACwAIABpAG4AIAB0AGgAZQAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAKQAgAHcAaABlAG4ALgAuAC4AIAB0AGgAZQAgAGwAYQBuAGQAIABpAHMAIABpAHIAcgBpAGcAYQB0AGUAZAAgACgAZQB4AGMAZQBwAHQAIABkAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgApAC4AJwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAJwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAJwAgAHQAbwAgAHMAaQBuAGcAdQBsAGEAcgAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQAnACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAPAAxACAAbQBvAG4AdABoAFwAIgAsACAAXAAiAEQAZQBlAHAAIABMAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAATQBhAG4AdQByAGUAIAAoAHcAaQB0AGgALwB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAIABpAG4AdABvACAAcABlAGwAbABlAHQAaQB6AGUAZAAgAGYAZQByAHQAaQBsAGkAcwBlAHIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUALAAgAFIAYQBuAGcAZQAgAGEAbgBkACAAUABhAGQAZABvAGMAawAgACgAYwApACgAZAApAFwAIgAsACAAXAAiAE0AQQBUACAAcgBhAHcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIxADAAXAAiACwAIAAwAC4ANgA2ACwAIAAwAC4AMQAsACAAMAAuADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAxACwAIAAwAC4ANgA4ACwAIAAwAC4AMQAsACAAMAAuADEAMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADIALAAgADAALgA3ACwAIAAwAC4AMQAsACAAMAAuADEAMwAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADMALAAgADAALgA3ADEALAAgADAALgAxACwAIAAwAC4AMQA0ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEANAAsACAAMAAuADcAMwAsACAAMAAuADEALAAgADAALgAxADUALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANQAsACAAMAAuADcANAAsACAAMAAuADEALAAgADAALgAxADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADYALAAgADAALgA3ADUALAAgADAALgAxACwAIAAwAC4AMQA4ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA3ACwAIAAwAC4ANwA2ACwAIAAwAC4AMQAsACAAMAAuADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADgALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA5ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMAAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADYALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADEALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA5ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAyACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADMAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMwAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADQALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA1ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADQAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAMgA2ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADQANAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAMgA3ACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA0ADgALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIjIAOABcACIALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADUALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBEAGkAZwBlAHMAdABlAHIAIAAvACAAYwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAHMAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBQAGkAdAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAE0AQQBUACAAcgBhAHcAXAAiACAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIAByAG8AdwAgAG8AZgAgAE4ASQBSACAATQBNAEEAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABEAHUAcABsAGkAYwBhAHQAZQBkACAAJwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgACcATQBBAFQAIAByAGEAdwAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgACYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIAAmACAARQBGAE4AMgBPAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -11903,18 +11166,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11933,7 +11196,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
@@ -11941,21 +11204,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>